<commit_message>
Pass 4 (mobile) batch 1: functional gaps from commcare-android Connect source
25 functional gaps (MTP vs code): behaviours present in the Connect/PersonalID
source with no MTP case - email OTP flow, Play Integrity attestation, duplicate/
country/rate-limit error paths, profile editing, launch retry, release toggles,
messaging encryption/offline queue, periodic notif retrieval. Plus 5 unit-test-
coverage observations for the dev-team deliverable. Covers the manager/network/
controller layer; fragment UI-validation + DB layers are the next sub-batches.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -1884,7 +1884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:J169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -8020,6 +8020,1326 @@
       <c r="J139" s="166" t="inlineStr">
         <is>
           <t>Pass 1 (mobile): MTP vs test suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-01</t>
+        </is>
+      </c>
+      <c r="B140" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Email</t>
+        </is>
+      </c>
+      <c r="C140" s="166" t="inlineStr">
+        <is>
+          <t>Email OTP collection: app offers to collect + verify an email after login (EmailOfferHelper), with sendEmailOtp/verifyEmailOtp endpoints</t>
+        </is>
+      </c>
+      <c r="D140" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E140" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP - entire email-OTP path absent. Real email round-trip. Src: EmailOfferHelper.kt, ApiPersonalId.sendEmailOtp/verifyEmailOtp</t>
+        </is>
+      </c>
+      <c r="F140" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G140" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H140" s="166" t="inlineStr"/>
+      <c r="I140" s="166" t="inlineStr"/>
+      <c r="J140" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-02</t>
+        </is>
+      </c>
+      <c r="B141" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Email</t>
+        </is>
+      </c>
+      <c r="C141" s="166" t="inlineStr">
+        <is>
+          <t>Email offer cadence: offered at most twice, second offer only after 30 days, skipped if email already set or toggle off</t>
+        </is>
+      </c>
+      <c r="D141" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E141" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Logic-level, unit-testable (EmailOfferHelperTest exists). Src: EmailOfferHelper.shouldOfferEmail</t>
+        </is>
+      </c>
+      <c r="F141" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G141" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H141" s="166" t="inlineStr"/>
+      <c r="I141" s="166" t="inlineStr"/>
+      <c r="J141" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-03</t>
+        </is>
+      </c>
+      <c r="B142" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C142" s="166" t="inlineStr">
+        <is>
+          <t>Device integrity / Play Integrity attestation during signup (reportIntegrity, startConfiguration; INTEGRITY_ERROR handling)</t>
+        </is>
+      </c>
+      <c r="D142" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E142" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Google Play Integrity infra. Src: ApiPersonalId.reportIntegrity/startConfiguration, PersonalIdApiHandler</t>
+        </is>
+      </c>
+      <c r="F142" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G142" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H142" s="166" t="inlineStr"/>
+      <c r="I142" s="166" t="inlineStr"/>
+      <c r="J142" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-04</t>
+        </is>
+      </c>
+      <c r="B143" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C143" s="166" t="inlineStr">
+        <is>
+          <t>Firebase ID token validation with phone match; PHONE_MISMATCH error when the token phone differs</t>
+        </is>
+      </c>
+      <c r="D143" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E143" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Firebase infra. Src: ApiPersonalId.validateFirebaseIdToken, PersonalIdApiHandler PHONE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="F143" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G143" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H143" s="166" t="inlineStr"/>
+      <c r="I143" s="166" t="inlineStr"/>
+      <c r="J143" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-05</t>
+        </is>
+      </c>
+      <c r="B144" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C144" s="166" t="inlineStr">
+        <is>
+          <t>Duplicate-account block: ACTIVE_USER_EXISTS error when signing up with a phone already tied to an active account</t>
+        </is>
+      </c>
+      <c r="D144" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E144" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (TC_18 covers fuzzy NAME dup, not phone). Src: PersonalIdApiHandler ACTIVE_USER_EXISTS</t>
+        </is>
+      </c>
+      <c r="F144" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G144" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H144" s="166" t="inlineStr"/>
+      <c r="I144" s="166" t="inlineStr"/>
+      <c r="J144" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-06</t>
+        </is>
+      </c>
+      <c r="B145" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C145" s="166" t="inlineStr">
+        <is>
+          <t>Unsupported-country / phone-not-validated block (UNSUPPORTED_COUNTRY, PHONE_NOT_VALIDATED -&gt; FORBIDDEN)</t>
+        </is>
+      </c>
+      <c r="D145" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E145" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdApiHandler UNSUPPORTED_COUNTRY/PHONE_NOT_VALIDATED</t>
+        </is>
+      </c>
+      <c r="F145" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G145" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H145" s="166" t="inlineStr"/>
+      <c r="I145" s="166" t="inlineStr"/>
+      <c r="J145" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-07</t>
+        </is>
+      </c>
+      <c r="B146" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C146" s="166" t="inlineStr">
+        <is>
+          <t>Uninvited-user OTP block: NOT_ALLOWED error when an uninvited user requests an OTP</t>
+        </is>
+      </c>
+      <c r="D146" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E146" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdApiHandler NOT_ALLOWED</t>
+        </is>
+      </c>
+      <c r="F146" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G146" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H146" s="166" t="inlineStr"/>
+      <c r="I146" s="166" t="inlineStr"/>
+      <c r="J146" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-08</t>
+        </is>
+      </c>
+      <c r="B147" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - OTP</t>
+        </is>
+      </c>
+      <c r="C147" s="166" t="inlineStr">
+        <is>
+          <t>Rate limiting: RATE_LIMITED error on too many OTP/auth attempts</t>
+        </is>
+      </c>
+      <c r="D147" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E147" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Server-timing dependent. Src: PersonalIdApiHandler RATE_LIMITED</t>
+        </is>
+      </c>
+      <c r="F147" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G147" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H147" s="166" t="inlineStr"/>
+      <c r="I147" s="166" t="inlineStr"/>
+      <c r="J147" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-09</t>
+        </is>
+      </c>
+      <c r="B148" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Photo</t>
+        </is>
+      </c>
+      <c r="C148" s="166" t="inlineStr">
+        <is>
+          <t>Photo upload errors: FILE_TOO_LARGE (photo exceeds server limit) and FAILED_TO_UPLOAD handling</t>
+        </is>
+      </c>
+      <c r="D148" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E148" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (TC_23-27 cover happy-path capture only). Src: PersonalIdApiHandler FILE_TOO_LARGE/FAILED_TO_UPLOAD</t>
+        </is>
+      </c>
+      <c r="F148" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G148" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H148" s="166" t="inlineStr"/>
+      <c r="I148" s="166" t="inlineStr"/>
+      <c r="J148" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-10</t>
+        </is>
+      </c>
+      <c r="B149" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Recovery</t>
+        </is>
+      </c>
+      <c r="C149" s="166" t="inlineStr">
+        <is>
+          <t>NO_RECOVERY_PIN_SET error path when recovering an account that never set a backup code</t>
+        </is>
+      </c>
+      <c r="D149" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E149" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdApiHandler NO_RECOVERY_PIN_SET</t>
+        </is>
+      </c>
+      <c r="F149" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G149" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H149" s="166" t="inlineStr"/>
+      <c r="I149" s="166" t="inlineStr"/>
+      <c r="J149" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-11</t>
+        </is>
+      </c>
+      <c r="B150" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - OTP</t>
+        </is>
+      </c>
+      <c r="C150" s="166" t="inlineStr">
+        <is>
+          <t>SMS User Consent auto-read: app auto-reads the incoming OTP SMS via Google consent dialog (SMSBroadcastReceiver / SmsRetriever)</t>
+        </is>
+      </c>
+      <c r="D150" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E150" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (only manual OTP entry covered). Real SMS. Src: SMSBroadcastReceiver.java</t>
+        </is>
+      </c>
+      <c r="F150" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G150" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H150" s="166" t="inlineStr"/>
+      <c r="I150" s="166" t="inlineStr"/>
+      <c r="J150" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-12</t>
+        </is>
+      </c>
+      <c r="B151" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Profile</t>
+        </is>
+      </c>
+      <c r="C151" s="166" t="inlineStr">
+        <is>
+          <t>Profile update: edit display name, photo, and secondary phone after account creation (updateProfile / secondary_phone)</t>
+        </is>
+      </c>
+      <c r="D151" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E151" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (creation covered, editing not). Src: ApiPersonalId.updateUserProfile</t>
+        </is>
+      </c>
+      <c r="F151" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G151" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H151" s="166" t="inlineStr"/>
+      <c r="I151" s="166" t="inlineStr"/>
+      <c r="J151" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-13</t>
+        </is>
+      </c>
+      <c r="B152" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C152" s="166" t="inlineStr">
+        <is>
+          <t>Device OS-version eligibility gate: signup requires Android 9 (SDK&gt;=P) via checkDeviceCompability</t>
+        </is>
+      </c>
+      <c r="D152" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E152" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_35 (which is no-fingerprint). OS-version gate distinct. Src: PersonalIdManager.checkDeviceCompability</t>
+        </is>
+      </c>
+      <c r="F152" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G152" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H152" s="166" t="inlineStr"/>
+      <c r="I152" s="166" t="inlineStr"/>
+      <c r="J152" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-14</t>
+        </is>
+      </c>
+      <c r="B153" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Startup</t>
+        </is>
+      </c>
+      <c r="C153" s="166" t="inlineStr">
+        <is>
+          <t>Corrupt-DB recovery: on broken Connect DB at init, user is shown PERSONALID_DB_STARTUP_ERROR global error</t>
+        </is>
+      </c>
+      <c r="D153" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E153" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Requires DB corruption. Src: PersonalIdManager.init / ConnectDatabaseHelper.isDbBroken</t>
+        </is>
+      </c>
+      <c r="F153" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G153" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H153" s="166" t="inlineStr"/>
+      <c r="I153" s="166" t="inlineStr"/>
+      <c r="J153" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-15</t>
+        </is>
+      </c>
+      <c r="B154" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Linking</t>
+        </is>
+      </c>
+      <c r="C154" s="166" t="inlineStr">
+        <is>
+          <t>Second link-to-PersonalID offer shown again after 30 days, capped at 2 offers</t>
+        </is>
+      </c>
+      <c r="D154" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E154" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (TC_36 covers first prompt only). Time-dependent. Src: PersonalIdManager.evaluateLinkOffer</t>
+        </is>
+      </c>
+      <c r="F154" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G154" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H154" s="166" t="inlineStr"/>
+      <c r="I154" s="166" t="inlineStr"/>
+      <c r="J154" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-16</t>
+        </is>
+      </c>
+      <c r="B155" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Linking</t>
+        </is>
+      </c>
+      <c r="C155" s="166" t="inlineStr">
+        <is>
+          <t>Delink prompt on password login: logging into a PersonalId-managed app with password prompts to sever the link (mobile-side)</t>
+        </is>
+      </c>
+      <c r="D155" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E155" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_40-42 (web/HQ side). Mobile delink dialog distinct. Src: PersonalIdManager.promptToDelinkPersonalIdApp</t>
+        </is>
+      </c>
+      <c r="F155" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G155" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H155" s="166" t="inlineStr"/>
+      <c r="I155" s="166" t="inlineStr"/>
+      <c r="J155" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-17</t>
+        </is>
+      </c>
+      <c r="B156" s="166" t="inlineStr">
+        <is>
+          <t>Connect - App Launch</t>
+        </is>
+      </c>
+      <c r="C156" s="166" t="inlineStr">
+        <is>
+          <t>Auto-login launch retry: learn/deliver launch retries up to 3 attempts then shows a persistent-error dialog</t>
+        </is>
+      </c>
+      <c r="D156" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E156" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (download/open covered, retry/failure not). Src: LaunchOutcomeRouter MAX_LAUNCH_ATTEMPTS=3</t>
+        </is>
+      </c>
+      <c r="F156" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G156" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H156" s="166" t="inlineStr"/>
+      <c r="I156" s="166" t="inlineStr"/>
+      <c r="J156" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-18</t>
+        </is>
+      </c>
+      <c r="B157" s="166" t="inlineStr">
+        <is>
+          <t>Connect - App Launch</t>
+        </is>
+      </c>
+      <c r="C157" s="166" t="inlineStr">
+        <is>
+          <t>App seat failure recovery: a seat failure routes the user back to DispatchActivity</t>
+        </is>
+      </c>
+      <c r="D157" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E157" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: LaunchOutcomeRouter AppSeatFailed / recoverFromSeatFailure</t>
+        </is>
+      </c>
+      <c r="F157" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G157" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H157" s="166" t="inlineStr"/>
+      <c r="I157" s="166" t="inlineStr"/>
+      <c r="J157" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-19</t>
+        </is>
+      </c>
+      <c r="B158" s="166" t="inlineStr">
+        <is>
+          <t>Connect - App Launch</t>
+        </is>
+      </c>
+      <c r="C158" s="166" t="inlineStr">
+        <is>
+          <t>Launch progress dialog states: Seating / Signing-in / Syncing (with %) shown during auto-login</t>
+        </is>
+      </c>
+      <c r="D158" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E158" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: LaunchProgressMapper / ConnectAppLaunchController</t>
+        </is>
+      </c>
+      <c r="F158" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G158" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H158" s="166" t="inlineStr"/>
+      <c r="I158" s="166" t="inlineStr"/>
+      <c r="J158" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-20</t>
+        </is>
+      </c>
+      <c r="B159" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Feature Flags</t>
+        </is>
+      </c>
+      <c r="C159" s="166" t="inlineStr">
+        <is>
+          <t>Release-toggle-gated behaviour: features enabled/disabled by server release toggles fetched periodically</t>
+        </is>
+      </c>
+      <c r="D159" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E159" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (no toggle-gated case). Src: ConnectReleaseTogglesWorker, ReleaseToggleHelper</t>
+        </is>
+      </c>
+      <c r="F159" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G159" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H159" s="166" t="inlineStr"/>
+      <c r="I159" s="166" t="inlineStr"/>
+      <c r="J159" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-21</t>
+        </is>
+      </c>
+      <c r="B160" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Deep Links</t>
+        </is>
+      </c>
+      <c r="C160" s="166" t="inlineStr">
+        <is>
+          <t>Generic-opportunity deep link resolves destination by job status (payments/delivery/learn/summary)</t>
+        </is>
+      </c>
+      <c r="D160" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E160" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: ConnectJobHelper.resolveGenericOpportunityDestination</t>
+        </is>
+      </c>
+      <c r="F160" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G160" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H160" s="166" t="inlineStr"/>
+      <c r="I160" s="166" t="inlineStr"/>
+      <c r="J160" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-22</t>
+        </is>
+      </c>
+      <c r="B161" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C161" s="166" t="inlineStr">
+        <is>
+          <t>Offline outgoing-message queue: unconfirmed outgoing messages are resent when connectivity returns</t>
+        </is>
+      </c>
+      <c r="D161" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E161" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Offline-dependent. Src: MessageManager.sendUnsentMessages</t>
+        </is>
+      </c>
+      <c r="F161" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G161" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H161" s="166" t="inlineStr"/>
+      <c r="I161" s="166" t="inlineStr"/>
+      <c r="J161" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-23</t>
+        </is>
+      </c>
+      <c r="B162" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C162" s="166" t="inlineStr">
+        <is>
+          <t>End-to-end message encryption: messages encrypted with channel key; send blocked if no encryption key present</t>
+        </is>
+      </c>
+      <c r="D162" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E162" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: MessageManager.sendMessage / ApiPersonalId.sendMessagingMessage (ciphertext/nonce/tag)</t>
+        </is>
+      </c>
+      <c r="F162" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G162" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H162" s="166" t="inlineStr"/>
+      <c r="I162" s="166" t="inlineStr"/>
+      <c r="J162" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-24</t>
+        </is>
+      </c>
+      <c r="B163" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Notifications</t>
+        </is>
+      </c>
+      <c r="C163" s="166" t="inlineStr">
+        <is>
+          <t>Periodic push-notification retrieval (polling, not just live push) scheduled on login, cancelled on logout</t>
+        </is>
+      </c>
+      <c r="D163" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E163" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (all notif cases are live-push). Src: NotificationsSyncWorkerManager, PersonalIdManager.userUnlockedPersonalId</t>
+        </is>
+      </c>
+      <c r="F163" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G163" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H163" s="166" t="inlineStr"/>
+      <c r="I163" s="166" t="inlineStr"/>
+      <c r="J163" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-25</t>
+        </is>
+      </c>
+      <c r="B164" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Background</t>
+        </is>
+      </c>
+      <c r="C164" s="166" t="inlineStr">
+        <is>
+          <t>Heartbeat worker: 4-hourly heartbeat refreshing FCM token, requires network + battery-not-low</t>
+        </is>
+      </c>
+      <c r="D164" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E164" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Background/time-dependent. Src: PersonalIdManager.scheduleHeartbeat, ConnectHeartbeatWorker</t>
+        </is>
+      </c>
+      <c r="F164" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G164" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H164" s="166" t="inlineStr"/>
+      <c r="I164" s="166" t="inlineStr"/>
+      <c r="J164" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="166" t="inlineStr">
+        <is>
+          <t>GAP-UTC-M-01</t>
+        </is>
+      </c>
+      <c r="B165" s="166" t="inlineStr">
+        <is>
+          <t>PersonalIdManager</t>
+        </is>
+      </c>
+      <c r="C165" s="166" t="inlineStr">
+        <is>
+          <t>No direct unit test for PersonalIdManager (status transitions, link/delink orchestration, token validity) despite it being the PersonalID workflow hub</t>
+        </is>
+      </c>
+      <c r="D165" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E165" s="166" t="inlineStr">
+        <is>
+          <t>Unit-test coverage gap. Src: connect/PersonalIdManager.java (656 lines)</t>
+        </is>
+      </c>
+      <c r="F165" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G165" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H165" s="166" t="inlineStr"/>
+      <c r="I165" s="166" t="inlineStr"/>
+      <c r="J165" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="166" t="inlineStr">
+        <is>
+          <t>GAP-UTC-M-02</t>
+        </is>
+      </c>
+      <c r="B166" s="166" t="inlineStr">
+        <is>
+          <t>MessageManager</t>
+        </is>
+      </c>
+      <c r="C166" s="166" t="inlineStr">
+        <is>
+          <t>No unit test for MessageManager (channel consent, encryption-key retrieval, unsent-message resend)</t>
+        </is>
+      </c>
+      <c r="D166" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E166" s="166" t="inlineStr">
+        <is>
+          <t>Unit-test coverage gap. Src: connect/MessageManager.java</t>
+        </is>
+      </c>
+      <c r="F166" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G166" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H166" s="166" t="inlineStr"/>
+      <c r="I166" s="166" t="inlineStr"/>
+      <c r="J166" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="166" t="inlineStr">
+        <is>
+          <t>GAP-UTC-M-03</t>
+        </is>
+      </c>
+      <c r="B167" s="166" t="inlineStr">
+        <is>
+          <t>ConnectSsoHelper</t>
+        </is>
+      </c>
+      <c r="C167" s="166" t="inlineStr">
+        <is>
+          <t>No unit test for ConnectSsoHelper (PersonalID/HQ token exchange + HQ-worker linking branches)</t>
+        </is>
+      </c>
+      <c r="D167" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E167" s="166" t="inlineStr">
+        <is>
+          <t>Unit-test coverage gap. Src: connect/network/ConnectSsoHelper.java</t>
+        </is>
+      </c>
+      <c r="F167" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G167" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H167" s="166" t="inlineStr"/>
+      <c r="I167" s="166" t="inlineStr"/>
+      <c r="J167" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="166" t="inlineStr">
+        <is>
+          <t>GAP-UTC-M-04</t>
+        </is>
+      </c>
+      <c r="B168" s="166" t="inlineStr">
+        <is>
+          <t>SMSBroadcastReceiver</t>
+        </is>
+      </c>
+      <c r="C168" s="166" t="inlineStr">
+        <is>
+          <t>No unit test for SMS consent receiver (success/timeout/error branches)</t>
+        </is>
+      </c>
+      <c r="D168" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E168" s="166" t="inlineStr">
+        <is>
+          <t>Unit-test coverage gap. Src: connect/SMSBroadcastReceiver.java</t>
+        </is>
+      </c>
+      <c r="F168" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G168" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H168" s="166" t="inlineStr"/>
+      <c r="I168" s="166" t="inlineStr"/>
+      <c r="J168" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="166" t="inlineStr">
+        <is>
+          <t>GAP-UTC-M-05</t>
+        </is>
+      </c>
+      <c r="B169" s="166" t="inlineStr">
+        <is>
+          <t>ApiPersonalId/ApiConnect</t>
+        </is>
+      </c>
+      <c r="C169" s="166" t="inlineStr">
+        <is>
+          <t>API request builders (params/headers/auth) exercised only via mock server, no per-endpoint builder unit tests</t>
+        </is>
+      </c>
+      <c r="D169" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E169" s="166" t="inlineStr">
+        <is>
+          <t>Unit-test coverage gap (partial). Src: connect/network/ApiPersonalId.java, ApiConnect.java</t>
+        </is>
+      </c>
+      <c r="F169" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G169" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H169" s="166" t="inlineStr"/>
+      <c r="I169" s="166" t="inlineStr"/>
+      <c r="J169" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
     </row>
@@ -8072,918 +9392,918 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>Personal ID Tests</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>TC_01</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>Confirm an existing user is able to sign in and is able to continue to work</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="0" t="inlineStr">
         <is>
           <t>test_tc_01 (existing demo-user sign-in)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>Personal ID Tests</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>TC_03</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>Verify user can logout of Personal ID and re-authenitcate themselves</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="0" t="inlineStr">
         <is>
           <t>test_tc_01 (forget PID / re-auth)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>Personal ID Tests</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>TC_28</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>Verify user is able to sign out, by clicking "Forget PersonalID user"</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>test_tc_01 (forget PersonalID sign out)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>Personal ID Tests</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>TC_31</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>Verify user is unable to recover the account, if they enter a wrong backup code</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>test_tc_01 (wrong backup code error)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="0" t="inlineStr">
         <is>
           <t>Personal ID Tests</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>TC_32</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>Verify user account is locked when they enter the backup code wrong more than 3 times</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>test_tc_02 (account locked popup)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>TC_01</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>Confirm after signing up with a Personal ID, user sees all the connect options in the side menu</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>test_tc_01 (connect side-menu options)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>TC_08</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>Verify on clicking the opportunities option from the side drawer takes you to the opportunity list page</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>test_tc_03 (opportunities option -&gt; list)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>TC_10</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>Verify on clicking the messaging option, user is taken channels list page</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>test_tc_07 (messaging -&gt; channels list)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>TC_17</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>Verify mobile users sess all the opportunities that they are invited to on the opportunity list page</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>test_tc_03 (opportunity list shown)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>TC_20</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>Verify on selecting the view opportunity button, user sees the description and all the opportunity details</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>test_tc_03 (view opportunity details/job card)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>TC_21</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>Ensure that after downloading the learn app, the opportunity status gets updated on the mobile</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>test_tc_04 (learn app in-progress status)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>TC_22</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>Verify user is able to dowload the Learn App from the opportunity</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>test_tc_04 (download learn app)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>TC_23</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>Ensure that user is taken to the app home screen after successful download of the Learn App</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>test_tc_04 (auto-login to learn app)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>TC_24</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>Verify on submitting the forms, learn app progress is updated in the app</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>test_tc_04 (learn progress updates)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>TC_26</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>Confirm user is unable to claim the job, if they don't pass the assessment</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>test_tc_04 (fail assessment - cannot claim)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>TC_27</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>Verify user can claim the job when they have successfully passed the assessment</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>test_tc_04 (pass assessment - certificate)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>TC_28</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>Confirm that user sees the Delivery details on the screen when they click on the "View Opportunity Details" button</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>test_tc_05 (claim job / delivery details)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>TC_29</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>Verify the number of visits is updated in the app after successfully conducting a visit</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>test_tc_05 (visits updated after submit)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>TC_30</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>Verify on approving a visit on connect web, the status is updated in the app as well</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="0" t="inlineStr">
         <is>
           <t>test_tc_05 (approve visit -&gt; status updates)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>TC_32</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>Verify user can only do the max visits allowed to them on a single day</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="0" t="inlineStr">
         <is>
           <t>test_tc_08 (max daily visits)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>TC_43</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>Verify that total amount paid to the user for the approved visits is displayed correctly under Payments tab</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="0" t="inlineStr">
         <is>
           <t>test_tc_06 (total paid amount on payments tab)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>TC_44</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>Verfiy user is able to see the payment transaction card on the payments tab</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="0" t="inlineStr">
         <is>
           <t>test_tc_06 (payment transaction card)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>TC_45</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>Verfiy user is not able to see the payment transaction card after clicking on ask later button</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="0" t="inlineStr">
         <is>
           <t>test_tc_06 (ask-later hides card)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="0" t="inlineStr">
         <is>
           <t>Integration Tests (Connect)</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>TC_46</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>Confirm that when a mobile user is suspended from an opportuntiy, the opportunity home page shows user suspended message</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="0" t="inlineStr">
         <is>
           <t>test_tc_07 (suspended-user message on app)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="0" t="inlineStr">
         <is>
           <t>Connect messaging</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>Connect message1</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>Verify user is able to create a broadcast with connect message option</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="0" t="inlineStr">
         <is>
           <t>test_tc_10 (broadcast connect message)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="0" t="inlineStr">
         <is>
           <t>Connect messaging</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>Connect message2</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>Verify user is able to create a broadcast with connect survey option</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="0" t="inlineStr">
         <is>
           <t>test_tc_10 (broadcast connect survey)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="0" t="inlineStr">
         <is>
           <t>Connect messaging</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>Connect message3</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>Verify user is able to create a Conditional alerts with connect message option</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="0" t="inlineStr">
         <is>
           <t>test_tc_09 (conditional alert connect message)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="0" t="inlineStr">
         <is>
           <t>Connect messaging</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>Connect message4</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>Verify user is able to create a conditional alerts with connect survey option</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="0" t="inlineStr">
         <is>
           <t>test_tc_09 (conditional alert connect survey)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="0" t="inlineStr">
         <is>
           <t>Connect Notifications</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>Notifications_01</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>Verify Notifications option is visible on left hand menu</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="0" t="inlineStr">
         <is>
           <t>test_tc_07 (notifications option on left menu)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="0" t="inlineStr">
         <is>
           <t>Connect Notifications</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>Notifications_02</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>Verify notiifcations icon is present on the opportunities list page</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="0" t="inlineStr">
         <is>
           <t>test_tc_03 (notifications icon on opp page)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="0" t="inlineStr">
         <is>
           <t>Connect Notifications</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>Notifications_04</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>Verify opportunity invite notification is shown on notifications history page</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="0" t="inlineStr">
         <is>
           <t>test_tc_03 (opp invite notification)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>Connect Notifications</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>Notifications_05</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>Verify we are able to land on opportunity's learn app upon clicking on the opportunity invite notification</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="0" t="inlineStr">
         <is>
           <t>test_tc_03 (land on learn app via notification)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>Connect Notifications</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
         <is>
           <t>Notifications_08</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>Verify Payment notifications are shown in notifications history page</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="0" t="inlineStr">
         <is>
           <t>test_tc_06 (payment notification)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="0" t="inlineStr">
         <is>
           <t>Connect Notifications</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
         <is>
           <t>Notifications_09</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>Verify user is able to land on the payment screen upon clicking on the payment notification</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="0" t="inlineStr">
         <is>
           <t>test_tc_06 (land on payment screen)</t>
         </is>

</xml_diff>

<commit_message>
Pass 4 (mobile) batch 2: fragment UI-layer functional gaps
12 functional gaps from the PersonalID signup fragments (GPS-location gating,
location/Play-Services/consent prerequisites, phone-hint autofill, dual OTP
provider fallback Firebase->Twilio, OTP rate-limit messages, PIN-vs-biometric
min-security + biometric error/enrollment states, name/backup-code validation).
Plus 3 cross-cutting: a MTP-vs-code discrepancy ('This is not me' marked
deprecated in MTP but still implemented) and 2 automation-enabler notes
(demo-user skips OTP; IS_QA_AUTOMATION build skips biometric).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -1884,7 +1884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J169"/>
+  <dimension ref="A1:J184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -9340,6 +9340,666 @@
       <c r="J169" s="166" t="inlineStr">
         <is>
           <t>Pass 4 (mobile): commcare-android Connect source</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-26</t>
+        </is>
+      </c>
+      <c r="B170" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C170" s="166" t="inlineStr">
+        <is>
+          <t>GPS location is MANDATORY to continue signup: continue button stays disabled until a location is acquired; screen shows 'using your location' / 'no location found' tooltip</t>
+        </is>
+      </c>
+      <c r="D170" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E170" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (TC_06 covers phone field only, not location gating). Src: PersonalIdPhoneFragment.allowedToContinue</t>
+        </is>
+      </c>
+      <c r="F170" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G170" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H170" s="166" t="inlineStr"/>
+      <c r="I170" s="166" t="inlineStr"/>
+      <c r="J170" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-27</t>
+        </is>
+      </c>
+      <c r="B171" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C171" s="166" t="inlineStr">
+        <is>
+          <t>Location permission / GPS-off handling: dedicated permission-error screens, GPS-settings resolution prompt, and 'grant location' recovery screens</t>
+        </is>
+      </c>
+      <c r="D171" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E171" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdPhoneFragment.onLocationRequestFailure / navigateToPermissionErrorMessageDisplay</t>
+        </is>
+      </c>
+      <c r="F171" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G171" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H171" s="166" t="inlineStr"/>
+      <c r="I171" s="166" t="inlineStr"/>
+      <c r="J171" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-28</t>
+        </is>
+      </c>
+      <c r="B172" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C172" s="166" t="inlineStr">
+        <is>
+          <t>Consent checkbox must be ticked before Continue is enabled on the phone screen</t>
+        </is>
+      </c>
+      <c r="D172" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E172" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdPhoneFragment.allowedToContinue (connectConsentCheck)</t>
+        </is>
+      </c>
+      <c r="F172" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G172" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H172" s="166" t="inlineStr"/>
+      <c r="I172" s="166" t="inlineStr"/>
+      <c r="J172" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-29</t>
+        </is>
+      </c>
+      <c r="B173" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C173" s="166" t="inlineStr">
+        <is>
+          <t>Google Play Services availability check on the phone screen; missing/outdated Play Services shows an update/resolution prompt and blocks signup</t>
+        </is>
+      </c>
+      <c r="D173" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E173" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdPhoneFragment.checkGooglePlayServices</t>
+        </is>
+      </c>
+      <c r="F173" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G173" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H173" s="166" t="inlineStr"/>
+      <c r="I173" s="166" t="inlineStr"/>
+      <c r="J173" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-30</t>
+        </is>
+      </c>
+      <c r="B174" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C174" s="166" t="inlineStr">
+        <is>
+          <t>Phone-number hint autofill: Google phone picker pre-fills country code + number on field focus</t>
+        </is>
+      </c>
+      <c r="D174" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E174" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdPhoneFragment.setupPhoneHintLauncher / displayPhoneNumber</t>
+        </is>
+      </c>
+      <c r="F174" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G174" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H174" s="166" t="inlineStr"/>
+      <c r="I174" s="166" t="inlineStr"/>
+      <c r="J174" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-31</t>
+        </is>
+      </c>
+      <c r="B175" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - OTP</t>
+        </is>
+      </c>
+      <c r="C175" s="166" t="inlineStr">
+        <is>
+          <t>Dual OTP provider with fallback: Firebase by default, auto-switches to Twilio (via PersonalID) on first resend or a non-recoverable Firebase error</t>
+        </is>
+      </c>
+      <c r="D175" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E175" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (no notion of two OTP providers). Real SMS across providers. Src: PersonalIdPhoneVerificationFragment.setupOtpManager/shouldAutoSwitchToPersonalIdAuth</t>
+        </is>
+      </c>
+      <c r="F175" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G175" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H175" s="166" t="inlineStr"/>
+      <c r="I175" s="166" t="inlineStr"/>
+      <c r="J175" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-32</t>
+        </is>
+      </c>
+      <c r="B176" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - OTP</t>
+        </is>
+      </c>
+      <c r="C176" s="166" t="inlineStr">
+        <is>
+          <t>OTP 'too many attempts' / verification-failed error messages (TOO_MANY_REQUESTS, VERIFICATION_FAILED, INVALID_CREDENTIAL)</t>
+        </is>
+      </c>
+      <c r="D176" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E176" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (TC_13 covers single wrong OTP only). Src: PersonalIdPhoneVerificationFragment otpCallback.onFailure</t>
+        </is>
+      </c>
+      <c r="F176" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G176" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H176" s="166" t="inlineStr"/>
+      <c r="I176" s="166" t="inlineStr"/>
+      <c r="J176" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-33</t>
+        </is>
+      </c>
+      <c r="B177" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Security</t>
+        </is>
+      </c>
+      <c r="C177" s="166" t="inlineStr">
+        <is>
+          <t>Minimum-security requirement (PIN vs BIOMETRIC) from session drives which of fingerprint/PIN options are shown and which is accepted</t>
+        </is>
+      </c>
+      <c r="D177" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E177" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdBiometricConfigFragment.updateUiBasedOnMinSecurityRequired</t>
+        </is>
+      </c>
+      <c r="F177" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G177" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H177" s="166" t="inlineStr"/>
+      <c r="I177" s="166" t="inlineStr"/>
+      <c r="J177" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-34</t>
+        </is>
+      </c>
+      <c r="B178" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Security</t>
+        </is>
+      </c>
+      <c r="C178" s="166" t="inlineStr">
+        <is>
+          <t>Biometric/PIN configuration error states: not-available, needs-update, no-hardware (distinct messages + retry vs fail)</t>
+        </is>
+      </c>
+      <c r="D178" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E178" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_35 (no-fingerprint only). Src: PersonalIdBiometricConfigFragment show*Error methods</t>
+        </is>
+      </c>
+      <c r="F178" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G178" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H178" s="166" t="inlineStr"/>
+      <c r="I178" s="166" t="inlineStr"/>
+      <c r="J178" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-35</t>
+        </is>
+      </c>
+      <c r="B179" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Security</t>
+        </is>
+      </c>
+      <c r="C179" s="166" t="inlineStr">
+        <is>
+          <t>Biometric enrollment-failed screen when the user cancels/leaves the device enrollment flow</t>
+        </is>
+      </c>
+      <c r="D179" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E179" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdBiometricConfigFragment.navigateToBiometricEnrollmentFailed</t>
+        </is>
+      </c>
+      <c r="F179" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G179" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H179" s="166" t="inlineStr"/>
+      <c r="I179" s="166" t="inlineStr"/>
+      <c r="J179" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-36</t>
+        </is>
+      </c>
+      <c r="B180" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C180" s="166" t="inlineStr">
+        <is>
+          <t>Name field validation: whitespace-only rejected, value trimmed before submit (continue disabled while blank)</t>
+        </is>
+      </c>
+      <c r="D180" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E180" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_17 (entry only). Src: PersonalIdNameFragment.createNameWatcher</t>
+        </is>
+      </c>
+      <c r="F180" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G180" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H180" s="166" t="inlineStr"/>
+      <c r="I180" s="166" t="inlineStr"/>
+      <c r="J180" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-37</t>
+        </is>
+      </c>
+      <c r="B181" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Recovery</t>
+        </is>
+      </c>
+      <c r="C181" s="166" t="inlineStr">
+        <is>
+          <t>Backup code auto-submits when the 6th digit is entered (code-complete listener), no explicit continue tap needed</t>
+        </is>
+      </c>
+      <c r="D181" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E181" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdBackupCodeFragment setCodeCompleteListener</t>
+        </is>
+      </c>
+      <c r="F181" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G181" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H181" s="166" t="inlineStr"/>
+      <c r="I181" s="166" t="inlineStr"/>
+      <c r="J181" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="166" t="inlineStr">
+        <is>
+          <t>GAP-MMISC-07</t>
+        </is>
+      </c>
+      <c r="B182" s="166" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="C182" s="166" t="inlineStr">
+        <is>
+          <t>DISCREPANCY: MTP TC_30 marks the 'This is not me' recovery option as deprecated, but the code still implements it (notMeButton -&gt; handleNotMeButtonPressed). Reconcile MTP vs app.</t>
+        </is>
+      </c>
+      <c r="D182" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E182" s="166" t="inlineStr">
+        <is>
+          <t>MTP-vs-code discrepancy found in pass 4. Src: PersonalIdBackupCodeFragment.handleNotMeButtonPressed</t>
+        </is>
+      </c>
+      <c r="F182" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G182" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H182" s="166" t="inlineStr"/>
+      <c r="I182" s="166" t="inlineStr"/>
+      <c r="J182" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="166" t="inlineStr">
+        <is>
+          <t>GAP-MMISC-08</t>
+        </is>
+      </c>
+      <c r="B183" s="166" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="C183" s="166" t="inlineStr">
+        <is>
+          <t>Automation enabler: a demo-user (test number) SKIPS the phone-OTP step entirely (biometric config snackbar -&gt; name screen). Explains how the suite automates signup; document so real-OTP path isn't assumed covered.</t>
+        </is>
+      </c>
+      <c r="D183" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E183" s="166" t="inlineStr">
+        <is>
+          <t>Automation/coverage note. Src: PersonalIdBiometricConfigFragment.navigateForward (getDemoUser)</t>
+        </is>
+      </c>
+      <c r="F183" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G183" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H183" s="166" t="inlineStr"/>
+      <c r="I183" s="166" t="inlineStr"/>
+      <c r="J183" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="166" t="inlineStr">
+        <is>
+          <t>GAP-MMISC-09</t>
+        </is>
+      </c>
+      <c r="B184" s="166" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="C184" s="166" t="inlineStr">
+        <is>
+          <t>Automation enabler: IS_QA_AUTOMATION build variant SKIPS biometric setup (phone success -&gt; name screen directly). Real biometric-config path is not exercised by automation.</t>
+        </is>
+      </c>
+      <c r="D184" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E184" s="166" t="inlineStr">
+        <is>
+          <t>Automation/coverage note. Src: PersonalIdPhoneFragment.onConfigurationSuccess (BuildConfig.IS_QA_AUTOMATION)</t>
+        </is>
+      </c>
+      <c r="F184" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G184" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H184" s="166" t="inlineStr"/>
+      <c r="I184" s="166" t="inlineStr"/>
+      <c r="J184" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pass 4 (mobile) batch 3: delivery/learn/messaging fragment gaps
13 functional gaps from the Connect delivery-progress, learn-progress, job-intro,
app-download and messaging fragments: payment-confirmation-tile 7-day re-show +
revoke, learn certificate/status/button-state detail, app-download failure &
verification paths, messaging input-disabled-when-unsubscribed, 30s in-chat
polling, optimistic send. Mobile Gap Analysis now 64 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -2851,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -5159,6 +5159,578 @@
       <c r="J52" s="166" t="inlineStr">
         <is>
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-38</t>
+        </is>
+      </c>
+      <c r="B53" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Delivery</t>
+        </is>
+      </c>
+      <c r="C53" s="166" t="inlineStr">
+        <is>
+          <t>Payment-confirmation tile: shows aggregate unconfirmed amount; 'No' hides it for 7 days then it reappears; only shown when network available</t>
+        </is>
+      </c>
+      <c r="D53" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E53" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_44/45 (which cover the card only). 7-day re-show + aggregate + offline-gating missing. Src: ConnectDeliveryProgressFragment.updatePaymentConfirmationTile</t>
+        </is>
+      </c>
+      <c r="F53" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G53" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H53" s="166" t="inlineStr"/>
+      <c r="I53" s="166" t="inlineStr"/>
+      <c r="J53" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-39</t>
+        </is>
+      </c>
+      <c r="B54" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Delivery</t>
+        </is>
+      </c>
+      <c r="C54" s="166" t="inlineStr">
+        <is>
+          <t>Revoke a confirmed payment: a payment marked received can be reverted via 'revoke transferred' dialog</t>
+        </is>
+      </c>
+      <c r="D54" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E54" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (TC_44/45 cover confirm only). Src: ConnectResultsSummaryListFragment PaymentViewHolder (llRevertPayment)</t>
+        </is>
+      </c>
+      <c r="F54" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G54" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H54" s="166" t="inlineStr"/>
+      <c r="I54" s="166" t="inlineStr"/>
+      <c r="J54" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-40</t>
+        </is>
+      </c>
+      <c r="B55" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Delivery</t>
+        </is>
+      </c>
+      <c r="C55" s="166" t="inlineStr">
+        <is>
+          <t>Delivery progress has Progress + Payment tabs; a notification/deep-link can open directly on the Payment tab</t>
+        </is>
+      </c>
+      <c r="D55" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E55" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs MTP. Tab structure + deep-link-to-payment-tab not asserted. Src: ConnectDeliveryProgressFragment.setupTabViewPager (initialTabPosition)</t>
+        </is>
+      </c>
+      <c r="F55" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G55" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H55" s="166" t="inlineStr"/>
+      <c r="I55" s="166" t="inlineStr"/>
+      <c r="J55" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-41</t>
+        </is>
+      </c>
+      <c r="B56" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Delivery</t>
+        </is>
+      </c>
+      <c r="C56" s="166" t="inlineStr">
+        <is>
+          <t>Delivery card message is colour-coded by state: complete (amber warning), relearn-tasks-completed (green), otherwise orange warning</t>
+        </is>
+      </c>
+      <c r="D56" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E56" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_49/50. Colour-state logic not covered. Src: ConnectDeliveryProgressFragment.updateCardMessage</t>
+        </is>
+      </c>
+      <c r="F56" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G56" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H56" s="166" t="inlineStr"/>
+      <c r="I56" s="166" t="inlineStr"/>
+      <c r="J56" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-42</t>
+        </is>
+      </c>
+      <c r="B57" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Learn</t>
+        </is>
+      </c>
+      <c r="C57" s="166" t="inlineStr">
+        <is>
+          <t>Certificate card shows subject, worker name and completion date once learning is complete AND assessment passed</t>
+        </is>
+      </c>
+      <c r="D57" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E57" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_27. Certificate detail fields not covered. Src: ConnectLearningProgressFragment.updateCertificateView</t>
+        </is>
+      </c>
+      <c r="F57" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G57" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H57" s="166" t="inlineStr"/>
+      <c r="I57" s="166" t="inlineStr"/>
+      <c r="J57" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-43</t>
+        </is>
+      </c>
+      <c r="B58" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Learn</t>
+        </is>
+      </c>
+      <c r="C58" s="166" t="inlineStr">
+        <is>
+          <t>Learn status messaging: passed/failed shows score vs passing score; 'needs assessment'; 'not started'; in-progress 'X of Y modules'</t>
+        </is>
+      </c>
+      <c r="D58" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E58" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_24-27. Distinct status strings/score display not covered. Src: ConnectLearningProgressFragment.getLearningStatus</t>
+        </is>
+      </c>
+      <c r="F58" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G58" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H58" s="166" t="inlineStr"/>
+      <c r="I58" s="166" t="inlineStr"/>
+      <c r="J58" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-44</t>
+        </is>
+      </c>
+      <c r="B59" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Learn</t>
+        </is>
+      </c>
+      <c r="C59" s="166" t="inlineStr">
+        <is>
+          <t>Learn button 4-state logic: Continue learning / Go to assessment / Download / View details, chosen by progress + app-installed state</t>
+        </is>
+      </c>
+      <c r="D59" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E59" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (only download/continue implied). Src: ConnectLearningProgressFragment.updateButtons</t>
+        </is>
+      </c>
+      <c r="F59" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G59" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H59" s="166" t="inlineStr"/>
+      <c r="I59" s="166" t="inlineStr"/>
+      <c r="J59" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-45</t>
+        </is>
+      </c>
+      <c r="B60" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Learn</t>
+        </is>
+      </c>
+      <c r="C60" s="166" t="inlineStr">
+        <is>
+          <t>'Learning ended' message shown when the opportunity has finished (project end date passed)</t>
+        </is>
+      </c>
+      <c r="D60" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E60" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: ConnectLearningProgressFragment.updateLearningStatus (job.isFinished)</t>
+        </is>
+      </c>
+      <c r="F60" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G60" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H60" s="166" t="inlineStr"/>
+      <c r="I60" s="166" t="inlineStr"/>
+      <c r="J60" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-46</t>
+        </is>
+      </c>
+      <c r="B61" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Download</t>
+        </is>
+      </c>
+      <c r="C61" s="166" t="inlineStr">
+        <is>
+          <t>App download failure handling: missing/invalid resource, incompatible-reqs -&gt; APK update prompt, target mismatch, duplicate-app -&gt; re-validate, unknown error; back disabled during install; post-download verification step</t>
+        </is>
+      </c>
+      <c r="D61" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E61" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_22 (basic download + back-disabled only). Failure/verification paths missing. Src: ConnectDownloadingFragment (Resource*Listener callbacks)</t>
+        </is>
+      </c>
+      <c r="F61" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G61" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H61" s="166" t="inlineStr"/>
+      <c r="I61" s="166" t="inlineStr"/>
+      <c r="J61" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-47</t>
+        </is>
+      </c>
+      <c r="B62" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Opportunity</t>
+        </is>
+      </c>
+      <c r="C62" s="166" t="inlineStr">
+        <is>
+          <t>Job intro details: multi-payment-unit breakdown vs single-payment text, 'no learning required' when no modules, days-remaining, max-daily-visits</t>
+        </is>
+      </c>
+      <c r="D62" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E62" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_20/28. Multi-payment/empty-module/limits detail not covered. Src: ConnectJobIntroFragment.buildPaymentText/populate*</t>
+        </is>
+      </c>
+      <c r="F62" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G62" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H62" s="166" t="inlineStr"/>
+      <c r="I62" s="166" t="inlineStr"/>
+      <c r="J62" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-48</t>
+        </is>
+      </c>
+      <c r="B63" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C63" s="166" t="inlineStr">
+        <is>
+          <t>Message input is disabled with a 'not subscribed' placeholder when the channel is unsubscribed; send icon appears only when text is entered AND the channel is subscribed</t>
+        </is>
+      </c>
+      <c r="D63" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E63" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: ConnectMessageFragment.setChannelUnsubscribedState / createTextWatcher</t>
+        </is>
+      </c>
+      <c r="F63" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G63" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H63" s="166" t="inlineStr"/>
+      <c r="I63" s="166" t="inlineStr"/>
+      <c r="J63" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-49</t>
+        </is>
+      </c>
+      <c r="B64" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C64" s="166" t="inlineStr">
+        <is>
+          <t>In-chat message polling every 30s while the chat screen is open (supplements push delivery)</t>
+        </is>
+      </c>
+      <c r="D64" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E64" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: ConnectMessageFragment apiCallRunnable (INTERVAL=30000)</t>
+        </is>
+      </c>
+      <c r="F64" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G64" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H64" s="166" t="inlineStr"/>
+      <c r="I64" s="166" t="inlineStr"/>
+      <c r="J64" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-50</t>
+        </is>
+      </c>
+      <c r="B65" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C65" s="166" t="inlineStr">
+        <is>
+          <t>Optimistic send: outgoing message shown immediately as unconfirmed, marked read on server ack; send-failure toast; empty-channel-list 'no channels' state</t>
+        </is>
+      </c>
+      <c r="D65" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E65" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: ConnectMessageFragment.sendMessage / ConnectMessageChannelListFragment.refreshUi</t>
+        </is>
+      </c>
+      <c r="F65" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G65" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H65" s="166" t="inlineStr"/>
+      <c r="I65" s="166" t="inlineStr"/>
+      <c r="J65" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pass 4 (mobile) batch 4: activities-layer gaps; mobile source read complete
5 functional gaps from activities/connect: feature-flag-gated notification bell,
logged-out deep-link guard, message-notification channel-resolution edge cases,
Work History earned+pending tabs, app-lock re-unlock on re-entry. views/connect
skimmed (custom view widgets, no functional behaviour). DB layer = data-model
reference only. Mobile pass-4 source analysis complete; Gap Analysis at 69 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -2851,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -5731,6 +5731,226 @@
       <c r="J65" s="166" t="inlineStr">
         <is>
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-51</t>
+        </is>
+      </c>
+      <c r="B66" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Notifications</t>
+        </is>
+      </c>
+      <c r="C66" s="166" t="inlineStr">
+        <is>
+          <t>Notification bell is feature-flag gated: it only appears when the NOTIFICATIONS feature flag is enabled</t>
+        </is>
+      </c>
+      <c r="D66" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E66" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (Notifications tab assumes always-present). Src: ConnectActivity.onCreateOptionsMenu (PersonalIdFeatureFlagChecker NOTIFICATIONS)</t>
+        </is>
+      </c>
+      <c r="F66" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G66" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H66" s="166" t="inlineStr"/>
+      <c r="I66" s="166" t="inlineStr"/>
+      <c r="J66" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-52</t>
+        </is>
+      </c>
+      <c r="B67" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Notifications</t>
+        </is>
+      </c>
+      <c r="C67" s="166" t="inlineStr">
+        <is>
+          <t>Logged-out deep-link guard: tapping a Connect/messaging notification while not signed into PersonalID shows an error toast and redirects to PersonalID signup</t>
+        </is>
+      </c>
+      <c r="D67" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E67" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: ConnectActivity/ConnectMessagingActivity onCreate (isloggedIn false branch)</t>
+        </is>
+      </c>
+      <c r="F67" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G67" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H67" s="166" t="inlineStr"/>
+      <c r="I67" s="166" t="inlineStr"/>
+      <c r="J67" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-53</t>
+        </is>
+      </c>
+      <c r="B68" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C68" s="166" t="inlineStr">
+        <is>
+          <t>Message-notification deep-link resolution: channel missing from local DB -&gt; network fetch; still missing -&gt; 'wrong channel' error; unconsented -&gt; channel list for consent; missing encryption key -&gt; fetch key first</t>
+        </is>
+      </c>
+      <c r="D68" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E68" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: ConnectMessagingActivity.handleChannelForValidity/handleNoChannel/checkForChannelEncryptionKey</t>
+        </is>
+      </c>
+      <c r="F68" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G68" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H68" s="166" t="inlineStr"/>
+      <c r="I68" s="166" t="inlineStr"/>
+      <c r="J68" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-54</t>
+        </is>
+      </c>
+      <c r="B69" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Worker History</t>
+        </is>
+      </c>
+      <c r="C69" s="166" t="inlineStr">
+        <is>
+          <t>Work History has Earned + Pending tabs: Pending (installed-app credentials not yet earned) is feature-flag gated (WORK_HISTORY_PENDING_TAB); earned sorted by issued-date desc; tab bar hidden when only one page</t>
+        </is>
+      </c>
+      <c r="D69" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E69" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs Worker_History tab (earned badges only). Pending tab / flag / sorting missing. Src: PersonalIdWorkHistoryActivity + PersonalIdWorkHistoryViewModel</t>
+        </is>
+      </c>
+      <c r="F69" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G69" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H69" s="166" t="inlineStr"/>
+      <c r="I69" s="166" t="inlineStr"/>
+      <c r="J69" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="166" t="inlineStr">
+        <is>
+          <t>GAP-SRC-M-55</t>
+        </is>
+      </c>
+      <c r="B70" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Security</t>
+        </is>
+      </c>
+      <c r="C70" s="166" t="inlineStr">
+        <is>
+          <t>App-lock re-unlock on re-entry: returning to Connect or opening from a message notification requires a PersonalID unlock (biometric/PIN) per unlock policy (e.g. session-with-time-threshold)</t>
+        </is>
+      </c>
+      <c r="D70" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E70" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: ConnectMessagingActivity (PersonalIdUnlocker.unlock) / connect_unlock_fragment</t>
+        </is>
+      </c>
+      <c r="F70" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G70" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H70" s="166" t="inlineStr"/>
+      <c r="I70" s="166" t="inlineStr"/>
+      <c r="J70" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pass 5 (mobile): frontend/config layer; mobile stream complete
6 gaps from the nav graph, feature-flag definitions, manifest, deep-link handler
and network interceptors: SMS invite deep-link handling + URI validation, the
feature-flag matrix (work_history_pending_tab and manage_profile currently OFF -
profile-editing not live, descope candidate), Connect data-load network/timeout/
parse error UX, POST_NOTIFICATIONS runtime prompt, API version-header contract.
Mobile passes 1/4/5 all complete; Gap Analysis at 75 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -2851,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -5951,6 +5951,270 @@
       <c r="J70" s="166" t="inlineStr">
         <is>
           <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="166" t="inlineStr">
+        <is>
+          <t>GAP-FE-M-01</t>
+        </is>
+      </c>
+      <c r="B71" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Deep Links</t>
+        </is>
+      </c>
+      <c r="C71" s="166" t="inlineStr">
+        <is>
+          <t>SMS invite deep link: app handles https://&lt;connect_host&gt;/users/invite_redirect/&lt;opp_uuid&gt; VIEW intents and routes to that opportunity; strict scheme/host/path validation; silently ignored (with analytics) if not signed in</t>
+        </is>
+      </c>
+      <c r="D71" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E71" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_18/19 (web-redirect side only). App-side URI handling + validation + logged-out ignore missing. Src: connect/utils/DeepLinkHelper.kt</t>
+        </is>
+      </c>
+      <c r="F71" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G71" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H71" s="166" t="inlineStr"/>
+      <c r="I71" s="166" t="inlineStr"/>
+      <c r="J71" s="166" t="inlineStr">
+        <is>
+          <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="166" t="inlineStr">
+        <is>
+          <t>GAP-FE-M-02</t>
+        </is>
+      </c>
+      <c r="B72" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Feature Flags</t>
+        </is>
+      </c>
+      <c r="C72" s="166" t="inlineStr">
+        <is>
+          <t>Feature-flag matrix untested: client flags work_history (on), work_history_pending_tab (OFF), notifications (on), manage_profile (OFF) + server toggle email_otp_verification gate whole features; MTP has no flag-state coverage - behaviours should be tested per state / current defaults documented</t>
+        </is>
+      </c>
+      <c r="D72" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E72" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PersonalIdFeatureFlagChecker.kt, ReleaseToggleHelper.kt</t>
+        </is>
+      </c>
+      <c r="F72" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G72" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H72" s="166" t="inlineStr"/>
+      <c r="I72" s="166" t="inlineStr"/>
+      <c r="J72" s="166" t="inlineStr">
+        <is>
+          <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="166" t="inlineStr">
+        <is>
+          <t>GAP-FE-M-03</t>
+        </is>
+      </c>
+      <c r="B73" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Feature Flags</t>
+        </is>
+      </c>
+      <c r="C73" s="166" t="inlineStr">
+        <is>
+          <t>manage_profile flag is currently OFF -&gt; profile management/editing (see GAP-SRC-M-12) is NOT live in the app today; treat as not-yet-shipped (descope/park until the flag is enabled)</t>
+        </is>
+      </c>
+      <c r="D73" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E73" s="166" t="inlineStr">
+        <is>
+          <t>Descope candidate - feature gated off. Src: PersonalIdFeatureFlagChecker MANAGE_PROFILE=false</t>
+        </is>
+      </c>
+      <c r="F73" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G73" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H73" s="166" t="inlineStr"/>
+      <c r="I73" s="166" t="inlineStr"/>
+      <c r="J73" s="166" t="inlineStr">
+        <is>
+          <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="166" t="inlineStr">
+        <is>
+          <t>GAP-FE-M-04</t>
+        </is>
+      </c>
+      <c r="B74" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Reliability</t>
+        </is>
+      </c>
+      <c r="C74" s="166" t="inlineStr">
+        <is>
+          <t>Connect data-load failure UX: opportunity/learn/delivery fetches surface network-error, 30s-timeout and JSON-parse-error states; no offline/error-path case in the MTP for Connect data loads</t>
+        </is>
+      </c>
+      <c r="D74" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E74" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: ConnectNetworkClient.executeApiCall / BaseApiClient (30s timeouts)</t>
+        </is>
+      </c>
+      <c r="F74" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G74" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H74" s="166" t="inlineStr"/>
+      <c r="I74" s="166" t="inlineStr"/>
+      <c r="J74" s="166" t="inlineStr">
+        <is>
+          <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="166" t="inlineStr">
+        <is>
+          <t>GAP-FE-M-05</t>
+        </is>
+      </c>
+      <c r="B75" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Notifications</t>
+        </is>
+      </c>
+      <c r="C75" s="166" t="inlineStr">
+        <is>
+          <t>POST_NOTIFICATIONS runtime permission prompt (Android 13+) is required to receive Connect push notifications</t>
+        </is>
+      </c>
+      <c r="D75" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E75" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: AndroidManifest POST_NOTIFICATIONS</t>
+        </is>
+      </c>
+      <c r="F75" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G75" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H75" s="166" t="inlineStr"/>
+      <c r="I75" s="166" t="inlineStr"/>
+      <c r="J75" s="166" t="inlineStr">
+        <is>
+          <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="166" t="inlineStr">
+        <is>
+          <t>GAP-FE-M-06</t>
+        </is>
+      </c>
+      <c r="B76" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Reliability</t>
+        </is>
+      </c>
+      <c r="C76" s="166" t="inlineStr">
+        <is>
+          <t>API version-header contract: client sends 'Accept: application/json;version=&lt;n&gt;' on Connect/PersonalID calls (server version negotiation)</t>
+        </is>
+      </c>
+      <c r="D76" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E76" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (infra). Src: BaseApiClient interceptor / ConnectNetworkHelper.addVersionHeader</t>
+        </is>
+      </c>
+      <c r="F76" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G76" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H76" s="166" t="inlineStr"/>
+      <c r="I76" s="166" t="inlineStr"/>
+      <c r="J76" s="166" t="inlineStr">
+        <is>
+          <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pass 4 (backend): connect-id PersonalID service gaps
15 backend functional gaps mapped to the mobile PersonalID/Connect surface:
multi-step account recovery (secondary phone / PIN / password reset), account
deactivation, change phone/password, payment phone profile, credential
issuance+accept flow, login-from-different-device detection, GPS->country
eligibility, device-integrity verdict breakdown, manual OTP, DB-key management,
session-token lifecycle. Plus a MTP-vs-backend discrepancy (OTP resend is
exponential backoff, not the fixed 120s the MTP states). Read urls/models/tasks/
auth/flags/payments; users/views.py + messaging views are an optional deeper
sub-pass. Mobile Gap Analysis now 91 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -2851,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -6215,6 +6215,710 @@
       <c r="J76" s="166" t="inlineStr">
         <is>
           <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-01</t>
+        </is>
+      </c>
+      <c r="B77" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Recovery</t>
+        </is>
+      </c>
+      <c r="C77" s="166" t="inlineStr">
+        <is>
+          <t>Multi-step account recovery state machine: primary-phone -&gt; secondary-phone -&gt; reset-password steps (RecoveryStatus). MTP covers only backup-code recovery</t>
+        </is>
+      </c>
+      <c r="D77" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E77" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (TC_29-32 = backup code only). Src: users/urls.py recover/* + RecoveryStatus model</t>
+        </is>
+      </c>
+      <c r="F77" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G77" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H77" s="166" t="inlineStr"/>
+      <c r="I77" s="166" t="inlineStr"/>
+      <c r="J77" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-02</t>
+        </is>
+      </c>
+      <c r="B78" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Recovery</t>
+        </is>
+      </c>
+      <c r="C78" s="166" t="inlineStr">
+        <is>
+          <t>Account recovery alternatives: recover via recovery PIN (confirm_recovery_pin), via backup code, and via password reset (reset_password/confirm_password)</t>
+        </is>
+      </c>
+      <c r="D78" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E78" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: users/views recover/confirm_pin, reset_password, confirm_password</t>
+        </is>
+      </c>
+      <c r="F78" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G78" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H78" s="166" t="inlineStr"/>
+      <c r="I78" s="166" t="inlineStr"/>
+      <c r="J78" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-03</t>
+        </is>
+      </c>
+      <c r="B79" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Phone</t>
+        </is>
+      </c>
+      <c r="C79" s="166" t="inlineStr">
+        <is>
+          <t>Secondary / recovery phone number: add + OTP-verify (validate_secondary_phone, confirm_secondary_otp) and recover via secondary phone</t>
+        </is>
+      </c>
+      <c r="D79" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E79" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: users/urls validate_secondary_phone / recover/secondary</t>
+        </is>
+      </c>
+      <c r="F79" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G79" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H79" s="166" t="inlineStr"/>
+      <c r="I79" s="166" t="inlineStr"/>
+      <c r="J79" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-04</t>
+        </is>
+      </c>
+      <c r="B80" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Account</t>
+        </is>
+      </c>
+      <c r="C80" s="166" t="inlineStr">
+        <is>
+          <t>Account deactivation: irreversible, confirmed via an SMS token valid 600s (initiate_deactivation / confirm_deactivation)</t>
+        </is>
+      </c>
+      <c r="D80" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="E80" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Real SMS + irreversible. Src: ConnectUser.initiate_deactivation</t>
+        </is>
+      </c>
+      <c r="F80" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G80" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H80" s="166" t="inlineStr"/>
+      <c r="I80" s="166" t="inlineStr"/>
+      <c r="J80" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-05</t>
+        </is>
+      </c>
+      <c r="B81" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Account</t>
+        </is>
+      </c>
+      <c r="C81" s="166" t="inlineStr">
+        <is>
+          <t>Change phone number (change_phone) and change password (change_password) for an existing account</t>
+        </is>
+      </c>
+      <c r="D81" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E81" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: users/urls change_phone / change_password</t>
+        </is>
+      </c>
+      <c r="F81" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G81" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H81" s="166" t="inlineStr"/>
+      <c r="I81" s="166" t="inlineStr"/>
+      <c r="J81" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-06</t>
+        </is>
+      </c>
+      <c r="B82" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Payments</t>
+        </is>
+      </c>
+      <c r="C82" s="166" t="inlineStr">
+        <is>
+          <t>Payment phone profile: worker sets a payment phone (with telecom-provider lookup) + OTP verify; PM approves/rejects/pends it, each state pushing a notification to the worker</t>
+        </is>
+      </c>
+      <c r="D82" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E82" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: payments/views.py (update_payment_profile_phone, ValidatePhoneNumbers)</t>
+        </is>
+      </c>
+      <c r="F82" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G82" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H82" s="166" t="inlineStr"/>
+      <c r="I82" s="166" t="inlineStr"/>
+      <c r="J82" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-07</t>
+        </is>
+      </c>
+      <c r="B83" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Credentials</t>
+        </is>
+      </c>
+      <c r="C83" s="166" t="inlineStr">
+        <is>
+          <t>Credential issuance &amp; acceptance: credential granted -&gt; SMS invite link -&gt; accept_credential; types APP_ACTIVITY/LEARN/DELIVER, levels, issuing authority (CONNECT/HQ x prod/staging/india)</t>
+        </is>
+      </c>
+      <c r="D83" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E83" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs Worker_History (earned display only). Invite/accept flow + types missing. Src: users/models Credential/UserCredential.add_credential</t>
+        </is>
+      </c>
+      <c r="F83" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G83" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H83" s="166" t="inlineStr"/>
+      <c r="I83" s="166" t="inlineStr"/>
+      <c r="J83" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-08</t>
+        </is>
+      </c>
+      <c r="B84" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C84" s="166" t="inlineStr">
+        <is>
+          <t>Phone-availability pre-check (phone_available) before starting signup</t>
+        </is>
+      </c>
+      <c r="D84" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E84" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: users/urls phone_available</t>
+        </is>
+      </c>
+      <c r="F84" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G84" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H84" s="166" t="inlineStr"/>
+      <c r="I84" s="166" t="inlineStr"/>
+      <c r="J84" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-09</t>
+        </is>
+      </c>
+      <c r="B85" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Security</t>
+        </is>
+      </c>
+      <c r="C85" s="166" t="inlineStr">
+        <is>
+          <t>Login-from-different-device detection: authenticating from a new device returns LOGIN_FROM_DIFFERENT_DEVICE; device last-accessed tracking (UserDeviceInfo)</t>
+        </is>
+      </c>
+      <c r="D85" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E85" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: users/auth.py DeviceBasicAuthentication / device_utils</t>
+        </is>
+      </c>
+      <c r="F85" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G85" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H85" s="166" t="inlineStr"/>
+      <c r="I85" s="166" t="inlineStr"/>
+      <c r="J85" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-10</t>
+        </is>
+      </c>
+      <c r="B86" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C86" s="166" t="inlineStr">
+        <is>
+          <t>GPS-derived country eligibility: signup GPS reverse-geocoded (MapBox) to a country code used for country restriction; ConfigurationSession expires after 4h</t>
+        </is>
+      </c>
+      <c r="D86" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E86" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (explains UNSUPPORTED_COUNTRY). Src: ConfigurationSession.country_code / is_valid</t>
+        </is>
+      </c>
+      <c r="F86" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G86" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H86" s="166" t="inlineStr"/>
+      <c r="I86" s="166" t="inlineStr"/>
+      <c r="J86" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-11</t>
+        </is>
+      </c>
+      <c r="B87" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C87" s="166" t="inlineStr">
+        <is>
+          <t>Device integrity verdict breakdown stored server-side: request-check, app-integrity, device-integrity, account-details sub-checks (DeviceIntegritySample); demo/test numbers bypass</t>
+        </is>
+      </c>
+      <c r="D87" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E87" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: users/models DeviceIntegritySample + report_integrity view</t>
+        </is>
+      </c>
+      <c r="F87" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G87" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H87" s="166" t="inlineStr"/>
+      <c r="I87" s="166" t="inlineStr"/>
+      <c r="J87" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-12</t>
+        </is>
+      </c>
+      <c r="B88" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - OTP</t>
+        </is>
+      </c>
+      <c r="C88" s="166" t="inlineStr">
+        <is>
+          <t>Manual OTP generation endpoint (generate_manual_otp) for support / when SMS auto-read fails; has_manual_otp monitoring flag</t>
+        </is>
+      </c>
+      <c r="D88" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E88" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: users/urls generate_manual_otp / SessionPhoneDevice.has_manual_otp</t>
+        </is>
+      </c>
+      <c r="F88" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G88" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H88" s="166" t="inlineStr"/>
+      <c r="I88" s="166" t="inlineStr"/>
+      <c r="J88" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-13</t>
+        </is>
+      </c>
+      <c r="B89" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Security</t>
+        </is>
+      </c>
+      <c r="C89" s="166" t="inlineStr">
+        <is>
+          <t>Local DB encryption key management: fetch_db_key issues/rotates a per-user key (UserKey valid flag); returned only after successful auth/backup-code</t>
+        </is>
+      </c>
+      <c r="D89" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E89" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: users/urls fetch_db_key / UserKey model</t>
+        </is>
+      </c>
+      <c r="F89" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G89" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H89" s="166" t="inlineStr"/>
+      <c r="I89" s="166" t="inlineStr"/>
+      <c r="J89" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-14</t>
+        </is>
+      </c>
+      <c r="B90" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Security</t>
+        </is>
+      </c>
+      <c r="C90" s="166" t="inlineStr">
+        <is>
+          <t>Session-token lifecycle: configuration session token expires after 4h (TOKEN_EXPIRED); locked account blocked at auth (LOCKED_ACCOUNT); invalid token rejected</t>
+        </is>
+      </c>
+      <c r="D90" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E90" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_32 (lock only). Token-expiry / invalid-token paths missing. Src: users/auth.py SessionTokenAuthentication</t>
+        </is>
+      </c>
+      <c r="F90" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G90" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H90" s="166" t="inlineStr"/>
+      <c r="I90" s="166" t="inlineStr"/>
+      <c r="J90" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-15</t>
+        </is>
+      </c>
+      <c r="B91" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Security</t>
+        </is>
+      </c>
+      <c r="C91" s="166" t="inlineStr">
+        <is>
+          <t>Device-security default rule: invited users default to PIN, non-invited default to BIOMETRIC (get_device_security_requirement) - drives the min-security screen</t>
+        </is>
+      </c>
+      <c r="D91" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E91" s="166" t="inlineStr">
+        <is>
+          <t>Clarifies GAP-SRC-M-33; rule not stated in MTP. Src: ConnectUser.get_device_security_requirement</t>
+        </is>
+      </c>
+      <c r="F91" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G91" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H91" s="166" t="inlineStr"/>
+      <c r="I91" s="166" t="inlineStr"/>
+      <c r="J91" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="166" t="inlineStr">
+        <is>
+          <t>GAP-MMISC-10</t>
+        </is>
+      </c>
+      <c r="B92" s="166" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="C92" s="166" t="inlineStr">
+        <is>
+          <t>DISCREPANCY: MTP TC_11 states OTP resend is enabled after 120 seconds, but the backend uses EXPONENTIAL backoff (2^attempts minutes, OTP valid 30 min) with a RateLimitedError/retry_after. Reconcile the MTP wait rule against server behaviour.</t>
+        </is>
+      </c>
+      <c r="D92" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E92" s="166" t="inlineStr">
+        <is>
+          <t>MTP-vs-backend discrepancy found in connect-id. Src: users/models BaseOTPDevice._attempt_send</t>
+        </is>
+      </c>
+      <c r="F92" s="166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G92" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H92" s="166" t="inlineStr"/>
+      <c r="I92" s="166" t="inlineStr"/>
+      <c r="J92" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pass 4 (backend) detail: connect-id users/views.py request-validation rules
Read users/views.py (1155 lines) in full. 8 additional gaps: AI-based name
similarity (cultural context), 7-day secondary-phone validation deadline,
new-device 'previous device' warning on recovery, HQ-invite SMS deeplink +
trusted-host callback + anti-enumeration, invited-only session OTP + version-
driven sms_method, email uniqueness (EMAIL_ALREADY_IN_USE), deactivation OAuth
token revocation, change-phone guards. connect-id backend now fully read.
Mobile Gap Analysis at 99 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -2851,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J92"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -6919,6 +6919,358 @@
       <c r="J92" s="166" t="inlineStr">
         <is>
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-16</t>
+        </is>
+      </c>
+      <c r="B93" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Signup</t>
+        </is>
+      </c>
+      <c r="C93" s="166" t="inlineStr">
+        <is>
+          <t>check_name duplicate detection is AI-based (OpenChatStudio) using the phone's country as cultural context; for a user who already owns the number it assumes same-user, and for non-invited Connect users the AI result is not acted on</t>
+        </is>
+      </c>
+      <c r="D93" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E93" s="166" t="inlineStr">
+        <is>
+          <t>Refines TC_18 (fuzzy match). AI/cultural-context + owns-number logic not in MTP. Src: check_user_similarity</t>
+        </is>
+      </c>
+      <c r="F93" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G93" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H93" s="166" t="inlineStr"/>
+      <c r="I93" s="166" t="inlineStr"/>
+      <c r="J93" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-17</t>
+        </is>
+      </c>
+      <c r="B94" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Phone</t>
+        </is>
+      </c>
+      <c r="C94" s="166" t="inlineStr">
+        <is>
+          <t>Recovery/secondary phone has a 7-day validation deadline set at registration (recovery_phone_validation_deadline); cleared once validated</t>
+        </is>
+      </c>
+      <c r="D94" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E94" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: register / confirm_secondary_otp</t>
+        </is>
+      </c>
+      <c r="F94" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G94" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H94" s="166" t="inlineStr"/>
+      <c r="I94" s="166" t="inlineStr"/>
+      <c r="J94" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-18</t>
+        </is>
+      </c>
+      <c r="B95" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Security</t>
+        </is>
+      </c>
+      <c r="C95" s="166" t="inlineStr">
+        <is>
+          <t>Backup-code recovery from a NEW device returns a 'previous_device' + last_accessed warning when the prior device was recently active (within threshold)</t>
+        </is>
+      </c>
+      <c r="D95" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E95" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (relates to GAP-BE-M-09). Src: confirm_backup_code (previous_device branch)</t>
+        </is>
+      </c>
+      <c r="F95" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G95" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H95" s="166" t="inlineStr"/>
+      <c r="I95" s="166" t="inlineStr"/>
+      <c r="J95" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-19</t>
+        </is>
+      </c>
+      <c r="B96" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - HQ Link</t>
+        </is>
+      </c>
+      <c r="C96" s="166" t="inlineStr">
+        <is>
+          <t>HQ invite flow: HQ forwards an invite -&gt; ConnectID sends an SMS deep link (connectid.dimagi.com/hq_invite) -&gt; confirm callback restricted to TRUSTED_COMMCAREHQ_HOSTS; unknown phone numbers get a fake-success (no user enumeration)</t>
+        </is>
+      </c>
+      <c r="D96" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E96" s="166" t="inlineStr">
+        <is>
+          <t>PARTIAL vs TC_36-46 (mobile linking). Invite-SMS/callback + trusted-host + anti-enumeration missing. Src: ForwardHQInvite / ConfirmHQInviteCallback</t>
+        </is>
+      </c>
+      <c r="F96" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G96" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H96" s="166" t="inlineStr"/>
+      <c r="I96" s="166" t="inlineStr"/>
+      <c r="J96" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-20</t>
+        </is>
+      </c>
+      <c r="B97" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - OTP</t>
+        </is>
+      </c>
+      <c r="C97" s="166" t="inlineStr">
+        <is>
+          <t>Session OTP (send_session_otp/confirm_session_otp, the Twilio/PersonalID path) is restricted to invited users (NOT_ALLOWED otherwise); API version selects sms_method (V1 PERSONAL_ID for invited else FIREBASE; newer FIREBASE + otp_fallback flag)</t>
+        </is>
+      </c>
+      <c r="D97" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E97" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (backs GAP-SRC-M-31 dual-provider). Src: send_session_otp / start_device_configuration</t>
+        </is>
+      </c>
+      <c r="F97" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G97" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H97" s="166" t="inlineStr"/>
+      <c r="I97" s="166" t="inlineStr"/>
+      <c r="J97" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-21</t>
+        </is>
+      </c>
+      <c r="B98" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Email</t>
+        </is>
+      </c>
+      <c r="C98" s="166" t="inlineStr">
+        <is>
+          <t>Email OTP uniqueness: verifying an email already tied to another active user returns EMAIL_ALREADY_IN_USE; a pre-account verified email is stored on the session and attached at profile completion</t>
+        </is>
+      </c>
+      <c r="D98" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E98" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (adds to email-OTP gaps). Src: verify_email_otp</t>
+        </is>
+      </c>
+      <c r="F98" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G98" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H98" s="166" t="inlineStr"/>
+      <c r="I98" s="166" t="inlineStr"/>
+      <c r="J98" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-22</t>
+        </is>
+      </c>
+      <c r="B99" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Account</t>
+        </is>
+      </c>
+      <c r="C99" s="166" t="inlineStr">
+        <is>
+          <t>Account deactivation revokes all OAuth access + refresh tokens (in addition to setting is_active=False); token must match and be within its validity window</t>
+        </is>
+      </c>
+      <c r="D99" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E99" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (adds to GAP-BE-M-04). Src: confirm_deactivation</t>
+        </is>
+      </c>
+      <c r="F99" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G99" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H99" s="166" t="inlineStr"/>
+      <c r="I99" s="166" t="inlineStr"/>
+      <c r="J99" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-23</t>
+        </is>
+      </c>
+      <c r="B100" s="166" t="inlineStr">
+        <is>
+          <t>PersonalID - Phone</t>
+        </is>
+      </c>
+      <c r="C100" s="166" t="inlineStr">
+        <is>
+          <t>Change-phone guards: a validated phone number cannot be changed; the supplied old number must match the current one</t>
+        </is>
+      </c>
+      <c r="D100" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E100" s="166" t="inlineStr">
+        <is>
+          <t>Refines GAP-BE-M-05. Src: change_phone</t>
+        </is>
+      </c>
+      <c r="F100" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G100" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H100" s="166" t="inlineStr"/>
+      <c r="I100" s="166" t="inlineStr"/>
+      <c r="J100" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pass 4 (backend): connect-id messaging service; connect-id fully read
5 server-side messaging gaps: message delivery-status lifecycle + receipt
callbacks, dedup by message_id, 7-day retention, server-side resend of
undelivered messages, server-enforced channel consent. connect-id repo now
read in full (users/messaging/payments/flags). Mobile Gap Analysis at 104 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -2851,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:J105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -7271,6 +7271,226 @@
       <c r="J100" s="166" t="inlineStr">
         <is>
           <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-24</t>
+        </is>
+      </c>
+      <c r="B101" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C101" s="166" t="inlineStr">
+        <is>
+          <t>Message delivery-status lifecycle: PENDING -&gt; SENT_TO_SERVICE -&gt; DELIVERED -&gt; CONFIRMED_RECEIVED, with HMAC-signed receipt-confirmation callbacks back to the HQ messaging service</t>
+        </is>
+      </c>
+      <c r="D101" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E101" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: messaging MessageStatus + UpdateReceivedView / send_messages_to_service_and_mark_status</t>
+        </is>
+      </c>
+      <c r="F101" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G101" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H101" s="166" t="inlineStr"/>
+      <c r="I101" s="166" t="inlineStr"/>
+      <c r="J101" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id messaging service</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-25</t>
+        </is>
+      </c>
+      <c r="B102" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C102" s="166" t="inlineStr">
+        <is>
+          <t>Message deduplication by message_id: a duplicate message_id is rejected (MESSAGE_ID_ALREADY_EXISTS) / skipped in bulk create</t>
+        </is>
+      </c>
+      <c r="D102" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E102" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: SendServerConnectMessage / SendMobileConnectMessage</t>
+        </is>
+      </c>
+      <c r="F102" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G102" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H102" s="166" t="inlineStr"/>
+      <c r="I102" s="166" t="inlineStr"/>
+      <c r="J102" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id messaging service</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-26</t>
+        </is>
+      </c>
+      <c r="B103" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C103" s="166" t="inlineStr">
+        <is>
+          <t>Message retention: messages are deleted 7 days after they are received (scheduled task)</t>
+        </is>
+      </c>
+      <c r="D103" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E103" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: messaging/tasks.delete_old_messages (MESSAGE_RETENTION_DAYS=7)</t>
+        </is>
+      </c>
+      <c r="F103" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G103" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H103" s="166" t="inlineStr"/>
+      <c r="I103" s="166" t="inlineStr"/>
+      <c r="J103" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id messaging service</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-27</t>
+        </is>
+      </c>
+      <c r="B104" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C104" s="166" t="inlineStr">
+        <is>
+          <t>Server-side resend of undelivered messages: a periodic task re-pushes FCM for messages still unreceived (received is null)</t>
+        </is>
+      </c>
+      <c r="D104" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E104" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (server counterpart to mobile offline queue). Src: resend_notifications_for_undelivered_messages</t>
+        </is>
+      </c>
+      <c r="F104" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G104" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H104" s="166" t="inlineStr"/>
+      <c r="I104" s="166" t="inlineStr"/>
+      <c r="J104" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id messaging service</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="166" t="inlineStr">
+        <is>
+          <t>GAP-BE-M-28</t>
+        </is>
+      </c>
+      <c r="B105" s="166" t="inlineStr">
+        <is>
+          <t>Connect - Messaging</t>
+        </is>
+      </c>
+      <c r="C105" s="166" t="inlineStr">
+        <is>
+          <t>Consent enforcement server-side: a server-&gt;mobile message to an unconsented channel is rejected (NO_USER_CONSENT); a channel defaults to consent=True at creation and creation pushes a 'New Channel' FCM</t>
+        </is>
+      </c>
+      <c r="D105" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E105" s="166" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (server side of consent; mobile input-disable is GAP-SRC-M-48). Src: SendServerConnectMessage / CreateChannelView</t>
+        </is>
+      </c>
+      <c r="F105" s="166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G105" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H105" s="166" t="inlineStr"/>
+      <c r="I105" s="166" t="inlineStr"/>
+      <c r="J105" s="166" t="inlineStr">
+        <is>
+          <t>Pass 4 (backend): connect-id messaging service</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Eng Coverage cross-reference column to both Gap Analysis tabs
Per Cal: tag every gap with whether eng's own PR-run tests already cover it, so
QA avoids duplicating eng work. Heuristic: manual/red gaps = QA-owned (real
device/SMS/push - eng can't unit-test either); automatable/yellow = eng-covered
at logic layer (QA e2e only if critical journey); connect-id backend gaps =
eng-covered; UTC rows = eng GAP (dev deliverable); per-gap overrides where no
matching eng test found (audio transcription, catchment, flag admin, reports,
accept-invite). Best-guess pending Cal confirmation.

Mobile: 78 eng-logic / 11 QA-owned / 5 eng-GAP / 10 N/A.
Web: 34 eng-logic / 5 partial / 7 N/A.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -2851,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:K105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -2864,6 +2864,7 @@
     <col width="12" customWidth="1" style="145" min="8" max="8"/>
     <col width="40" customWidth="1" style="145" min="9" max="9"/>
     <col width="28" customWidth="1" style="145" min="10" max="10"/>
+    <col width="46" customWidth="1" style="145" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2917,6 +2918,11 @@
           <t>Source</t>
         </is>
       </c>
+      <c r="K1" s="165" t="inlineStr">
+        <is>
+          <t>Eng Coverage</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="166" t="inlineStr">
@@ -2961,6 +2967,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="K2" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="166" t="inlineStr">
@@ -3005,6 +3016,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="K3" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="166" t="inlineStr">
@@ -3049,6 +3065,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="K4" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="166" t="inlineStr">
@@ -3093,6 +3114,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="K5" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="166" t="inlineStr">
@@ -3137,6 +3163,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="K6" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="166" t="inlineStr">
@@ -3181,6 +3212,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="K7" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="166" t="inlineStr">
@@ -3225,6 +3261,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K8" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="166" t="inlineStr">
@@ -3269,6 +3310,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K9" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="166" t="inlineStr">
@@ -3313,6 +3359,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K10" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="166" t="inlineStr">
@@ -3357,6 +3408,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K11" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="166" t="inlineStr">
@@ -3401,6 +3457,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K12" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="166" t="inlineStr">
@@ -3445,6 +3506,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K13" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="166" t="inlineStr">
@@ -3489,6 +3555,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K14" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="166" t="inlineStr">
@@ -3533,6 +3604,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K15" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="166" t="inlineStr">
@@ -3577,6 +3653,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K16" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="166" t="inlineStr">
@@ -3621,6 +3702,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K17" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="166" t="inlineStr">
@@ -3665,6 +3751,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K18" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="166" t="inlineStr">
@@ -3709,6 +3800,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K19" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="166" t="inlineStr">
@@ -3753,6 +3849,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K20" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="166" t="inlineStr">
@@ -3797,6 +3898,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K21" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="166" t="inlineStr">
@@ -3841,6 +3947,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K22" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="166" t="inlineStr">
@@ -3885,6 +3996,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K23" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="166" t="inlineStr">
@@ -3929,6 +4045,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K24" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="166" t="inlineStr">
@@ -3973,6 +4094,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K25" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="166" t="inlineStr">
@@ -4017,6 +4143,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K26" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="166" t="inlineStr">
@@ -4061,6 +4192,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K27" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="166" t="inlineStr">
@@ -4105,6 +4241,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K28" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="166" t="inlineStr">
@@ -4149,6 +4290,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K29" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="166" t="inlineStr">
@@ -4193,6 +4339,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K30" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="166" t="inlineStr">
@@ -4237,6 +4388,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K31" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="166" t="inlineStr">
@@ -4281,6 +4437,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K32" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="166" t="inlineStr">
@@ -4325,6 +4486,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K33" s="166" t="inlineStr">
+        <is>
+          <t>Eng GAP (no unit test) - dev deliverable</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="166" t="inlineStr">
@@ -4369,6 +4535,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K34" s="166" t="inlineStr">
+        <is>
+          <t>Eng GAP (no unit test) - dev deliverable</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="166" t="inlineStr">
@@ -4413,6 +4584,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K35" s="166" t="inlineStr">
+        <is>
+          <t>Eng GAP (no unit test) - dev deliverable</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="166" t="inlineStr">
@@ -4457,6 +4633,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K36" s="166" t="inlineStr">
+        <is>
+          <t>Eng GAP (no unit test) - dev deliverable</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="166" t="inlineStr">
@@ -4501,6 +4682,11 @@
           <t>Pass 4 (mobile): commcare-android Connect source</t>
         </is>
       </c>
+      <c r="K37" s="166" t="inlineStr">
+        <is>
+          <t>Eng GAP (no unit test) - dev deliverable</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="166" t="inlineStr">
@@ -4545,6 +4731,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K38" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="166" t="inlineStr">
@@ -4589,6 +4780,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K39" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="166" t="inlineStr">
@@ -4633,6 +4829,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K40" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="166" t="inlineStr">
@@ -4677,6 +4878,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K41" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="166" t="inlineStr">
@@ -4721,6 +4927,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K42" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="166" t="inlineStr">
@@ -4765,6 +4976,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K43" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="166" t="inlineStr">
@@ -4809,6 +5025,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K44" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (real device/external; eng cannot unit-test)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="166" t="inlineStr">
@@ -4853,6 +5074,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K45" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="166" t="inlineStr">
@@ -4897,6 +5123,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K46" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="166" t="inlineStr">
@@ -4941,6 +5172,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K47" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="166" t="inlineStr">
@@ -4985,6 +5221,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K48" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="166" t="inlineStr">
@@ -5029,6 +5270,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K49" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="166" t="inlineStr">
@@ -5073,6 +5319,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K50" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="166" t="inlineStr">
@@ -5117,6 +5368,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K51" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="166" t="inlineStr">
@@ -5161,6 +5417,11 @@
           <t>Pass 4 (mobile) batch 2: fragment UI layer</t>
         </is>
       </c>
+      <c r="K52" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="166" t="inlineStr">
@@ -5205,6 +5466,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K53" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="166" t="inlineStr">
@@ -5249,6 +5515,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K54" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="166" t="inlineStr">
@@ -5293,6 +5564,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K55" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="166" t="inlineStr">
@@ -5337,6 +5613,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K56" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="166" t="inlineStr">
@@ -5381,6 +5662,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K57" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="166" t="inlineStr">
@@ -5425,6 +5711,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K58" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="166" t="inlineStr">
@@ -5469,6 +5760,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K59" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="166" t="inlineStr">
@@ -5513,6 +5809,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K60" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="166" t="inlineStr">
@@ -5557,6 +5858,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K61" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="166" t="inlineStr">
@@ -5601,6 +5907,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K62" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="166" t="inlineStr">
@@ -5645,6 +5956,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K63" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="166" t="inlineStr">
@@ -5689,6 +6005,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K64" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="166" t="inlineStr">
@@ -5733,6 +6054,11 @@
           <t>Pass 4 (mobile) batch 3: connect delivery/learn/messaging fragments</t>
         </is>
       </c>
+      <c r="K65" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="166" t="inlineStr">
@@ -5777,6 +6103,11 @@
           <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
         </is>
       </c>
+      <c r="K66" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="166" t="inlineStr">
@@ -5821,6 +6152,11 @@
           <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
         </is>
       </c>
+      <c r="K67" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="166" t="inlineStr">
@@ -5865,6 +6201,11 @@
           <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
         </is>
       </c>
+      <c r="K68" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="166" t="inlineStr">
@@ -5909,6 +6250,11 @@
           <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
         </is>
       </c>
+      <c r="K69" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="166" t="inlineStr">
@@ -5953,6 +6299,11 @@
           <t>Pass 4 (mobile) batch 4: activities/connect layer</t>
         </is>
       </c>
+      <c r="K70" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="166" t="inlineStr">
@@ -5997,6 +6348,11 @@
           <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
         </is>
       </c>
+      <c r="K71" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="166" t="inlineStr">
@@ -6041,6 +6397,11 @@
           <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
         </is>
       </c>
+      <c r="K72" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="166" t="inlineStr">
@@ -6085,6 +6446,11 @@
           <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
         </is>
       </c>
+      <c r="K73" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="166" t="inlineStr">
@@ -6129,6 +6495,11 @@
           <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
         </is>
       </c>
+      <c r="K74" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="166" t="inlineStr">
@@ -6173,6 +6544,11 @@
           <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
         </is>
       </c>
+      <c r="K75" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="166" t="inlineStr">
@@ -6217,6 +6593,11 @@
           <t>Pass 5 (mobile): nav/feature-flags/manifest/deep-links/interceptors</t>
         </is>
       </c>
+      <c r="K76" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="166" t="inlineStr">
@@ -6261,6 +6642,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K77" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="166" t="inlineStr">
@@ -6305,6 +6691,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K78" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="166" t="inlineStr">
@@ -6349,6 +6740,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K79" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="166" t="inlineStr">
@@ -6393,6 +6789,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K80" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="166" t="inlineStr">
@@ -6437,6 +6838,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K81" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="166" t="inlineStr">
@@ -6481,6 +6887,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K82" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="166" t="inlineStr">
@@ -6525,6 +6936,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K83" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="166" t="inlineStr">
@@ -6569,6 +6985,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K84" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="166" t="inlineStr">
@@ -6613,6 +7034,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K85" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="166" t="inlineStr">
@@ -6657,6 +7083,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K86" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="166" t="inlineStr">
@@ -6701,6 +7132,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K87" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="166" t="inlineStr">
@@ -6745,6 +7181,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K88" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="166" t="inlineStr">
@@ -6789,6 +7230,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K89" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="166" t="inlineStr">
@@ -6833,6 +7279,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K90" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="166" t="inlineStr">
@@ -6877,6 +7328,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K91" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="166" t="inlineStr">
@@ -6921,6 +7377,11 @@
           <t>Pass 4 (backend): connect-id (PersonalID service)</t>
         </is>
       </c>
+      <c r="K92" s="166" t="inlineStr">
+        <is>
+          <t>N/A (hygiene/discrepancy/automation note)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="166" t="inlineStr">
@@ -6965,6 +7426,11 @@
           <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
         </is>
       </c>
+      <c r="K93" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="166" t="inlineStr">
@@ -7009,6 +7475,11 @@
           <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
         </is>
       </c>
+      <c r="K94" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="166" t="inlineStr">
@@ -7053,6 +7524,11 @@
           <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
         </is>
       </c>
+      <c r="K95" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="166" t="inlineStr">
@@ -7097,6 +7573,11 @@
           <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
         </is>
       </c>
+      <c r="K96" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="166" t="inlineStr">
@@ -7141,6 +7622,11 @@
           <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
         </is>
       </c>
+      <c r="K97" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="166" t="inlineStr">
@@ -7185,6 +7671,11 @@
           <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
         </is>
       </c>
+      <c r="K98" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="166" t="inlineStr">
@@ -7229,6 +7720,11 @@
           <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
         </is>
       </c>
+      <c r="K99" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="166" t="inlineStr">
@@ -7273,6 +7769,11 @@
           <t>Pass 4 (backend): connect-id users/views.py (detail sub-pass)</t>
         </is>
       </c>
+      <c r="K100" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="166" t="inlineStr">
@@ -7317,6 +7818,11 @@
           <t>Pass 4 (backend): connect-id messaging service</t>
         </is>
       </c>
+      <c r="K101" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="166" t="inlineStr">
@@ -7361,6 +7867,11 @@
           <t>Pass 4 (backend): connect-id messaging service</t>
         </is>
       </c>
+      <c r="K102" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="166" t="inlineStr">
@@ -7405,6 +7916,11 @@
           <t>Pass 4 (backend): connect-id messaging service</t>
         </is>
       </c>
+      <c r="K103" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="166" t="inlineStr">
@@ -7449,6 +7965,11 @@
           <t>Pass 4 (backend): connect-id messaging service</t>
         </is>
       </c>
+      <c r="K104" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="166" t="inlineStr">
@@ -7491,6 +8012,11 @@
       <c r="J105" s="166" t="inlineStr">
         <is>
           <t>Pass 4 (backend): connect-id messaging service</t>
+        </is>
+      </c>
+      <c r="K105" s="166" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Extend Shubham's unit-test-coverage dimension to web (+ connect-id note)
Symmetry across streams: Cal's eng-coverage cross-ref already on both; Shubham's
unit-test-coverage-GAP dimension was mobile(android)-only. Added 5 web UTC gaps
(GAP-UTC-W-*): oauth2_validator (security), commcarehq views, flags admin layer,
microplanning forms, user signals. Both eng suites are strong so the lists are
deliberately short (good-news finding). Added 1 connect-id note (UTC-M-06):
backend well-covered except the connectid project app. Tagged Eng Coverage=GAP.
Web 51 rows, Mobile 105 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -2851,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -8017,6 +8017,55 @@
       <c r="K105" s="166" t="inlineStr">
         <is>
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="166" t="inlineStr">
+        <is>
+          <t>GAP-UTC-M-06</t>
+        </is>
+      </c>
+      <c r="B106" s="166" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="C106" s="166" t="inlineStr">
+        <is>
+          <t>connect-id backend is well unit-tested (users/messaging/payments have test suites); the only thin spot is the connectid project app (connectid/views.py + project config) which has no tests</t>
+        </is>
+      </c>
+      <c r="D106" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E106" s="166" t="inlineStr">
+        <is>
+          <t>Unit-test coverage note (connect-id) - completes mobile UTC symmetry. Src: connectid/views.py</t>
+        </is>
+      </c>
+      <c r="F106" s="166" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G106" s="166" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H106" s="166" t="inlineStr"/>
+      <c r="I106" s="166" t="inlineStr"/>
+      <c r="J106" s="166" t="inlineStr">
+        <is>
+          <t>connect-id: unit-test-coverage note</t>
+        </is>
+      </c>
+      <c r="K106" s="166" t="inlineStr">
+        <is>
+          <t>Eng GAP (no unit test) - dev deliverable</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make the two outputs explicit: Action column + Summary tab
Per Akanksha - separate the two deliverables. Action column on every Gap Analysis
row: 'Add to MTP only (eng-covered)' / 'Add to MTP + Automate (QA-owned)' /
'Add to MTP + Automate (confirm w/ eng)' / 'Dev: add unit test' / 'Reconcile'.
Summary tab with live COUNTIF formulas rolls up Output 1 (MTP completeness = all
128 functional gaps), Output 2 (automation backlog = 16 not-eng-covered), the
112 eng-covered add-to-MTP-only items, dev unit-test gaps, and cross-cutting.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -4,18 +4,19 @@
   <workbookPr/>
   <sheets>
     <sheet name="Legend" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name=" Test Tracker" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Personal ID Tests" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Integration Tests (Connect)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Connect Landing Page" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Connect messaging" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Connect Notifications" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Connect worker History" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Case List map " sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Test Tracker Horizontal" sheetId="10" state="hidden" r:id="rId10"/>
-    <sheet name="Automation Status" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gap Analysis" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Automation Coverage" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name=" Test Tracker" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Personal ID Tests" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Integration Tests (Connect)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Connect Landing Page" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Connect messaging" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Connect Notifications" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Connect worker History" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Case List map " sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Test Tracker Horizontal" sheetId="11" state="hidden" r:id="rId11"/>
+    <sheet name="Automation Status" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Gap Analysis" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Automation Coverage" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -402,7 +403,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="169">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -848,6 +849,8 @@
     <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1504,6 +1507,426 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="19.63" customWidth="1" style="145" min="1" max="1"/>
+    <col width="36" customWidth="1" style="145" min="2" max="2"/>
+    <col width="47.38" customWidth="1" style="145" min="3" max="3"/>
+    <col width="46.38" customWidth="1" style="145" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="72" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B1" s="72" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steps </t>
+        </is>
+      </c>
+      <c r="D1" s="72" t="inlineStr">
+        <is>
+          <t>Expected Outcome</t>
+        </is>
+      </c>
+      <c r="E1" s="72" t="inlineStr">
+        <is>
+          <t>Status (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="F1" s="72" t="inlineStr">
+        <is>
+          <t>Ticket/ Bug ID</t>
+        </is>
+      </c>
+      <c r="G1" s="72" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="H1" s="101" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="162" t="inlineStr">
+        <is>
+          <t>Case List Map</t>
+        </is>
+      </c>
+      <c r="B2" s="150" t="n"/>
+      <c r="C2" s="150" t="n"/>
+      <c r="D2" s="150" t="n"/>
+      <c r="E2" s="150" t="n"/>
+      <c r="F2" s="150" t="n"/>
+      <c r="G2" s="151" t="n"/>
+      <c r="H2" s="66" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="96" t="inlineStr">
+        <is>
+          <t>Map_01</t>
+        </is>
+      </c>
+      <c r="B3" s="97" t="inlineStr">
+        <is>
+          <t>Verify user is able to configure geo options</t>
+        </is>
+      </c>
+      <c r="C3" s="97" t="inlineStr">
+        <is>
+          <t>1. Login to CC HQ
+2. Navigate to applications 
+3. select any case list application
+4. Navigate to case list settings 
+5. Go to case list tab
+6. Under display properties configure the geo boundary and geo points'
+Note: Geo boundary and geo points options are visible only when address property is configured</t>
+        </is>
+      </c>
+      <c r="D3" s="97" t="inlineStr">
+        <is>
+          <t>- Geo boundary and geopoints options are available only when address display property is added
+- Geo boundary colour is available when geo boundary options is configured
+- Geo points colour is available when geo points option is configured
+- When "Address" property is deleted , Geo boundary and geo points options are automatically removed and  "requires column with format: Address" message is dispalyed
+ - When geo boundary is deleted, geo boundary colour is automatically removed and message is displayed
+- When geo point is deleted, geo point colour is automatically removed and message is displayed</t>
+        </is>
+      </c>
+      <c r="E3" s="66" t="n"/>
+      <c r="F3" s="66" t="n"/>
+      <c r="G3" s="66" t="n"/>
+      <c r="H3" s="103" t="inlineStr">
+        <is>
+          <t>Refer these tests to configure case list map properties - https://docs.google.com/spreadsheets/d/1ENauf0cWqR0c9Seu29xarLucB78j3bNJzuQ7ut0T7Fs/edit?gid=2#gid=2&amp;range=18:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="96" t="inlineStr">
+        <is>
+          <t>Map_02</t>
+        </is>
+      </c>
+      <c r="B4" s="104" t="inlineStr">
+        <is>
+          <t>Verify removal of required Geo options</t>
+        </is>
+      </c>
+      <c r="C4" s="97" t="inlineStr">
+        <is>
+          <t>Continue to above TC:
+ - Remove address property, check informational message is displayed
+ Repeated the above step with geo boundary and geo points</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>- When "Address" property is deleted , Geo boundary and geo points options are automatically removed and  "requires column with format: Address" message is dispalyed
+ - When geo boundary is deleted, geo boundary colour is automatically removed and message is displayed
+- When geo point is deleted, geo point colour is automatically removed and message is displayed</t>
+        </is>
+      </c>
+      <c r="E4" s="66" t="n"/>
+      <c r="F4" s="66" t="n"/>
+      <c r="G4" s="66" t="n"/>
+      <c r="H4" s="66" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="96" t="inlineStr">
+        <is>
+          <t>Map_03</t>
+        </is>
+      </c>
+      <c r="B5" s="97" t="inlineStr">
+        <is>
+          <t>Verify polygons and points are displayed on the case list map</t>
+        </is>
+      </c>
+      <c r="C5" s="97" t="inlineStr">
+        <is>
+          <t>1. Install CCC app
+2. Install the app used in map_01
+3. Login to the app
+4. Submit few forms with boundary box and points data and colours in hex code
+5. Navigate to case list follow up form
+6. Click on three dots menu
+7. Click on view map</t>
+        </is>
+      </c>
+      <c r="D5" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Polygons as per submitted data and colors should get highligted on the map
+</t>
+        </is>
+      </c>
+      <c r="E5" s="66" t="n"/>
+      <c r="F5" s="66" t="n"/>
+      <c r="G5" s="66" t="n"/>
+      <c r="H5" s="66" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="96" t="inlineStr">
+        <is>
+          <t>Map_04</t>
+        </is>
+      </c>
+      <c r="B6" s="104" t="inlineStr">
+        <is>
+          <t>Verify multiple locations display correctly</t>
+        </is>
+      </c>
+      <c r="C6" s="97" t="inlineStr">
+        <is>
+          <t>1. Submit multiple forms with different locations
+2. Navigate to case list
+3. Click on 3 dots menu &gt;&gt; view on map</t>
+        </is>
+      </c>
+      <c r="D6" s="97" t="inlineStr">
+        <is>
+          <t>- Multiple polygonas and points are visible clearly on the map with their resspective submitted colors</t>
+        </is>
+      </c>
+      <c r="E6" s="66" t="n"/>
+      <c r="F6" s="66" t="n"/>
+      <c r="G6" s="66" t="n"/>
+      <c r="H6" s="66" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="96" t="inlineStr">
+        <is>
+          <t>Map_05</t>
+        </is>
+      </c>
+      <c r="B7" s="104" t="inlineStr">
+        <is>
+          <t>Verify overlapping polygons for same coordinates</t>
+        </is>
+      </c>
+      <c r="C7" s="97" t="inlineStr">
+        <is>
+          <t>1. Submit the 2 or 3 forms with same boundary and points details
+2.  Navigate to case list
+3. Click on 3 dots menu &gt;&gt; view on map</t>
+        </is>
+      </c>
+      <c r="D7" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Cases with same location get overlap on each other and only one case is highlighted </t>
+        </is>
+      </c>
+      <c r="E7" s="66" t="n"/>
+      <c r="F7" s="66" t="n"/>
+      <c r="G7" s="66" t="n"/>
+      <c r="H7" s="66" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="96" t="inlineStr">
+        <is>
+          <t>Map_06</t>
+        </is>
+      </c>
+      <c r="B8" s="104" t="inlineStr">
+        <is>
+          <t>Verify case name popup appears on clicking a polygon</t>
+        </is>
+      </c>
+      <c r="C8" s="105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+Click on a polygon on the map.</t>
+        </is>
+      </c>
+      <c r="D8" s="97" t="inlineStr">
+        <is>
+          <t>- Case name appears upon clicking on the polygon</t>
+        </is>
+      </c>
+      <c r="E8" s="66" t="n"/>
+      <c r="F8" s="66" t="n"/>
+      <c r="G8" s="66" t="n"/>
+      <c r="H8" s="66" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="96" t="inlineStr">
+        <is>
+          <t>Map_07</t>
+        </is>
+      </c>
+      <c r="B9" s="104" t="inlineStr">
+        <is>
+          <t>Verify user can open the Case Follow-Up form by clicking on case name</t>
+        </is>
+      </c>
+      <c r="C9" s="97" t="inlineStr">
+        <is>
+          <t>Click on the case name on the map</t>
+        </is>
+      </c>
+      <c r="D9" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> - User redirects to the case follow up form</t>
+        </is>
+      </c>
+      <c r="E9" s="66" t="n"/>
+      <c r="F9" s="66" t="n"/>
+      <c r="G9" s="66" t="n"/>
+      <c r="H9" s="66" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="96" t="inlineStr">
+        <is>
+          <t>Map_08</t>
+        </is>
+      </c>
+      <c r="B10" s="104" t="inlineStr">
+        <is>
+          <t>Verify warning message on the mobile map for wrong configuration</t>
+        </is>
+      </c>
+      <c r="C10" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Submit few forms with geo boundary and point details
+2. Few forms with out complete or incorrect details
+3. Navigate to case list form &gt;&gt; view on map
+</t>
+        </is>
+      </c>
+      <c r="D10" s="97" t="inlineStr">
+        <is>
+          <t>- User should see a below message at the bottom of screen 
+"There was an error in app configuration due to which not all markers on the map are loaded correctly.”</t>
+        </is>
+      </c>
+      <c r="E10" s="66" t="n"/>
+      <c r="F10" s="66" t="n"/>
+      <c r="G10" s="66" t="n"/>
+      <c r="H10" s="66" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="96" t="inlineStr">
+        <is>
+          <t>Map_09</t>
+        </is>
+      </c>
+      <c r="B11" s="104" t="inlineStr">
+        <is>
+          <t>Verify visibility of individual toggles based on entity count</t>
+        </is>
+      </c>
+      <c r="C11" s="97" t="inlineStr">
+        <is>
+          <t>1. Submit only one form with one entity either boundary box or points
+2. Navigate to case list map</t>
+        </is>
+      </c>
+      <c r="D11" s="97" t="inlineStr">
+        <is>
+          <t>- Toggle buttons are not visible and by default they are in "ON"
+-  toggle panel is hidden if less than two toggles are needed
+- Location should get highlighted as per your form submission</t>
+        </is>
+      </c>
+      <c r="E11" s="66" t="n"/>
+      <c r="F11" s="66" t="n"/>
+      <c r="G11" s="66" t="n"/>
+      <c r="H11" s="66" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="96" t="inlineStr">
+        <is>
+          <t>Map_10</t>
+        </is>
+      </c>
+      <c r="B12" s="104" t="inlineStr">
+        <is>
+          <t>Verify toggles are shown when multiple entities exist</t>
+        </is>
+      </c>
+      <c r="C12" s="97" t="inlineStr">
+        <is>
+          <t>1. Submit multiple forms with multiple entities
+2. Navigate to case list map</t>
+        </is>
+      </c>
+      <c r="D12" s="97" t="inlineStr">
+        <is>
+          <t>- Toggle buttons are visible
+- Entire toggle panel is shown if at least two toggles are needed</t>
+        </is>
+      </c>
+      <c r="E12" s="66" t="n"/>
+      <c r="F12" s="66" t="n"/>
+      <c r="G12" s="66" t="n"/>
+      <c r="H12" s="66" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="96" t="inlineStr">
+        <is>
+          <t>Map_11</t>
+        </is>
+      </c>
+      <c r="B13" s="104" t="inlineStr">
+        <is>
+          <t>Verify user can toggle polygons and points ON/OFF</t>
+        </is>
+      </c>
+      <c r="C13" s="97" t="inlineStr">
+        <is>
+          <t>continue to above TC:
+ - Toggle off the polygons button, ON the geo points
+ - Toggle off the geopoints button, On the polygons button
+ - Off both at a time</t>
+        </is>
+      </c>
+      <c r="D13" s="97" t="inlineStr">
+        <is>
+          <t>- By default polygons and geo points are ON
+- When user off the polyongs, boundary colour is not shown and only point is shown on map
+- When user off the geopoints, boundary is shown and point is not shown
+- When turn off both , neither points nor boundary are visible</t>
+        </is>
+      </c>
+      <c r="E13" s="66" t="n"/>
+      <c r="F13" s="66" t="n"/>
+      <c r="G13" s="66" t="n"/>
+      <c r="H13" s="66" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="E3:E13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,N/A,Blocking"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" location="gid=2&amp;range=18:23" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F593"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
@@ -6478,7 +6901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7444,13 +7867,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K106"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="145" min="1" max="1"/>
@@ -7464,6 +7887,7 @@
     <col width="40" customWidth="1" style="145" min="9" max="9"/>
     <col width="28" customWidth="1" style="145" min="10" max="10"/>
     <col width="46" customWidth="1" style="145" min="11" max="11"/>
+    <col width="40" customWidth="1" style="145" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7522,6 +7946,11 @@
           <t>Eng Coverage</t>
         </is>
       </c>
+      <c r="L1" s="165" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="166" t="inlineStr">
@@ -7571,6 +8000,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L2" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="166" t="inlineStr">
@@ -7620,6 +8054,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L3" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="166" t="inlineStr">
@@ -7669,6 +8108,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L4" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="166" t="inlineStr">
@@ -7718,6 +8162,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L5" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="166" t="inlineStr">
@@ -7767,6 +8216,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L6" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="166" t="inlineStr">
@@ -7816,6 +8270,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L7" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="166" t="inlineStr">
@@ -7865,6 +8324,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L8" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="166" t="inlineStr">
@@ -7914,6 +8378,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L9" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="166" t="inlineStr">
@@ -7963,6 +8432,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L10" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="166" t="inlineStr">
@@ -8012,6 +8486,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L11" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="166" t="inlineStr">
@@ -8061,6 +8540,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L12" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="166" t="inlineStr">
@@ -8110,6 +8594,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L13" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="166" t="inlineStr">
@@ -8159,6 +8648,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L14" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="166" t="inlineStr">
@@ -8208,6 +8702,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L15" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="166" t="inlineStr">
@@ -8257,6 +8756,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L16" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="166" t="inlineStr">
@@ -8306,6 +8810,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L17" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="166" t="inlineStr">
@@ -8355,6 +8864,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L18" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="166" t="inlineStr">
@@ -8404,6 +8918,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L19" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="166" t="inlineStr">
@@ -8453,6 +8972,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L20" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="166" t="inlineStr">
@@ -8502,6 +9026,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L21" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="166" t="inlineStr">
@@ -8551,6 +9080,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L22" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="166" t="inlineStr">
@@ -8600,6 +9134,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L23" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="166" t="inlineStr">
@@ -8649,6 +9188,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L24" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="166" t="inlineStr">
@@ -8698,6 +9242,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L25" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="166" t="inlineStr">
@@ -8747,6 +9296,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L26" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="166" t="inlineStr">
@@ -8796,6 +9350,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L27" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="166" t="inlineStr">
@@ -8845,6 +9404,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L28" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="166" t="inlineStr">
@@ -8894,6 +9458,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L29" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="166" t="inlineStr">
@@ -8943,6 +9512,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L30" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="166" t="inlineStr">
@@ -8992,6 +9566,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L31" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="166" t="inlineStr">
@@ -9041,6 +9620,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L32" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="166" t="inlineStr">
@@ -9090,6 +9674,11 @@
           <t>Eng GAP (no unit test) - dev deliverable</t>
         </is>
       </c>
+      <c r="L33" s="166" t="inlineStr">
+        <is>
+          <t>Dev: add unit test</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="166" t="inlineStr">
@@ -9139,6 +9728,11 @@
           <t>Eng GAP (no unit test) - dev deliverable</t>
         </is>
       </c>
+      <c r="L34" s="166" t="inlineStr">
+        <is>
+          <t>Dev: add unit test</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="166" t="inlineStr">
@@ -9188,6 +9782,11 @@
           <t>Eng GAP (no unit test) - dev deliverable</t>
         </is>
       </c>
+      <c r="L35" s="166" t="inlineStr">
+        <is>
+          <t>Dev: add unit test</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="166" t="inlineStr">
@@ -9237,6 +9836,11 @@
           <t>Eng GAP (no unit test) - dev deliverable</t>
         </is>
       </c>
+      <c r="L36" s="166" t="inlineStr">
+        <is>
+          <t>Dev: add unit test</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="166" t="inlineStr">
@@ -9286,6 +9890,11 @@
           <t>Eng GAP (no unit test) - dev deliverable</t>
         </is>
       </c>
+      <c r="L37" s="166" t="inlineStr">
+        <is>
+          <t>Dev: add unit test</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="166" t="inlineStr">
@@ -9335,6 +9944,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L38" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="166" t="inlineStr">
@@ -9384,6 +9998,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L39" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="166" t="inlineStr">
@@ -9433,6 +10052,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L40" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="166" t="inlineStr">
@@ -9482,6 +10106,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L41" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="166" t="inlineStr">
@@ -9531,6 +10160,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L42" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="166" t="inlineStr">
@@ -9580,6 +10214,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L43" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="166" t="inlineStr">
@@ -9629,6 +10268,11 @@
           <t>QA-owned (real device/external; eng cannot unit-test)</t>
         </is>
       </c>
+      <c r="L44" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="166" t="inlineStr">
@@ -9678,6 +10322,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L45" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="166" t="inlineStr">
@@ -9727,6 +10376,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L46" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="166" t="inlineStr">
@@ -9776,6 +10430,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L47" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="166" t="inlineStr">
@@ -9825,6 +10484,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L48" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="166" t="inlineStr">
@@ -9874,6 +10538,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L49" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="166" t="inlineStr">
@@ -9923,6 +10592,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L50" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="166" t="inlineStr">
@@ -9972,6 +10646,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L51" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="166" t="inlineStr">
@@ -10021,6 +10700,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L52" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="166" t="inlineStr">
@@ -10070,6 +10754,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L53" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="166" t="inlineStr">
@@ -10119,6 +10808,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L54" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="166" t="inlineStr">
@@ -10168,6 +10862,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L55" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="166" t="inlineStr">
@@ -10217,6 +10916,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L56" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="166" t="inlineStr">
@@ -10266,6 +10970,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L57" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="166" t="inlineStr">
@@ -10315,6 +11024,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L58" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="166" t="inlineStr">
@@ -10364,6 +11078,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L59" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="166" t="inlineStr">
@@ -10413,6 +11132,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L60" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="166" t="inlineStr">
@@ -10462,6 +11186,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L61" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="166" t="inlineStr">
@@ -10511,6 +11240,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L62" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="166" t="inlineStr">
@@ -10560,6 +11294,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L63" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="166" t="inlineStr">
@@ -10609,6 +11348,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L64" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="166" t="inlineStr">
@@ -10658,6 +11402,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L65" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="166" t="inlineStr">
@@ -10707,6 +11456,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L66" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="166" t="inlineStr">
@@ -10756,6 +11510,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L67" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="166" t="inlineStr">
@@ -10805,6 +11564,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L68" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="166" t="inlineStr">
@@ -10854,6 +11618,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L69" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="166" t="inlineStr">
@@ -10903,6 +11672,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L70" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="166" t="inlineStr">
@@ -10952,6 +11726,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L71" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="166" t="inlineStr">
@@ -11001,6 +11780,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L72" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="166" t="inlineStr">
@@ -11050,6 +11834,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L73" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="166" t="inlineStr">
@@ -11099,6 +11888,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L74" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="166" t="inlineStr">
@@ -11148,6 +11942,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L75" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="166" t="inlineStr">
@@ -11197,6 +11996,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L76" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="166" t="inlineStr">
@@ -11246,6 +12050,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L77" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="166" t="inlineStr">
@@ -11295,6 +12104,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L78" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="166" t="inlineStr">
@@ -11344,6 +12158,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L79" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="166" t="inlineStr">
@@ -11393,6 +12212,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L80" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="166" t="inlineStr">
@@ -11442,6 +12266,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L81" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="166" t="inlineStr">
@@ -11491,6 +12320,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L82" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="166" t="inlineStr">
@@ -11540,6 +12374,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L83" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="166" t="inlineStr">
@@ -11589,6 +12428,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L84" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="166" t="inlineStr">
@@ -11638,6 +12482,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L85" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="166" t="inlineStr">
@@ -11687,6 +12536,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L86" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="166" t="inlineStr">
@@ -11736,6 +12590,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L87" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="166" t="inlineStr">
@@ -11785,6 +12644,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L88" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="166" t="inlineStr">
@@ -11834,6 +12698,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L89" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="166" t="inlineStr">
@@ -11883,6 +12752,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L90" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="166" t="inlineStr">
@@ -11932,6 +12806,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L91" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="166" t="inlineStr">
@@ -11981,6 +12860,11 @@
           <t>N/A (hygiene/discrepancy/automation note)</t>
         </is>
       </c>
+      <c r="L92" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="166" t="inlineStr">
@@ -12030,6 +12914,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L93" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="166" t="inlineStr">
@@ -12079,6 +12968,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L94" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="166" t="inlineStr">
@@ -12128,6 +13022,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L95" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="166" t="inlineStr">
@@ -12177,6 +13076,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L96" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="166" t="inlineStr">
@@ -12226,6 +13130,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L97" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="166" t="inlineStr">
@@ -12275,6 +13184,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L98" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="166" t="inlineStr">
@@ -12324,6 +13238,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L99" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="166" t="inlineStr">
@@ -12373,6 +13292,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L100" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="166" t="inlineStr">
@@ -12422,6 +13346,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L101" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="166" t="inlineStr">
@@ -12471,6 +13400,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L102" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="166" t="inlineStr">
@@ -12520,6 +13454,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L103" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="166" t="inlineStr">
@@ -12569,6 +13508,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L104" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="166" t="inlineStr">
@@ -12618,6 +13562,11 @@
           <t>Eng-covered (logic) - QA e2e only if critical journey</t>
         </is>
       </c>
+      <c r="L105" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="166" t="inlineStr">
@@ -12665,6 +13614,11 @@
       <c r="K106" s="166" t="inlineStr">
         <is>
           <t>Eng GAP (no unit test) - dev deliverable</t>
+        </is>
+      </c>
+      <c r="L106" s="166" t="inlineStr">
+        <is>
+          <t>Dev: add unit test</t>
         </is>
       </c>
     </row>
@@ -12673,7 +13627,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18560,6 +19514,142 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="66" customWidth="1" style="145" min="1" max="1"/>
+    <col width="12" customWidth="1" style="145" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Gap Analysis — Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="170" t="inlineStr">
+        <is>
+          <t>OUTPUT 1 — MTP completeness (all functional gaps: add to the MTP)</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"Add to MTP*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ...of which already eng-covered (add to MTP only, do NOT automate)</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"Add to MTP only*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ...of which QA to automate (see Output 2)</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"*Automate*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="170" t="inlineStr">
+        <is>
+          <t>OUTPUT 2 — QA automation backlog (functional gaps NOT eng-covered)</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"*Automate*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   QA-owned (real device/SMS/push - eng cannot cover)</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"*QA-owned*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Automatable, confirm w/ eng (partial coverage)</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"*confirm w/ eng*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="170" t="inlineStr">
+        <is>
+          <t>DEV deliverable — unit-test-coverage gaps (eng to add unit tests)</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"Dev:*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="170" t="inlineStr">
+        <is>
+          <t>CROSS-CUTTING — reconcile plan/code (hygiene/discrepancy)</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"Reconcile*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="170" t="inlineStr">
+        <is>
+          <t>TOTAL Gap Analysis rows</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>COUNTA('Gap Analysis'!$L$2:$L$1000)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -19181,7 +20271,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFFFFF"/>
@@ -20465,7 +21555,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -22130,7 +23220,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -22984,7 +24074,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -23386,7 +24476,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -24004,7 +25094,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -24169,424 +25259,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="19.63" customWidth="1" style="145" min="1" max="1"/>
-    <col width="36" customWidth="1" style="145" min="2" max="2"/>
-    <col width="47.38" customWidth="1" style="145" min="3" max="3"/>
-    <col width="46.38" customWidth="1" style="145" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="72" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B1" s="72" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C1" s="72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Steps </t>
-        </is>
-      </c>
-      <c r="D1" s="72" t="inlineStr">
-        <is>
-          <t>Expected Outcome</t>
-        </is>
-      </c>
-      <c r="E1" s="72" t="inlineStr">
-        <is>
-          <t>Status (Pass/Fail)</t>
-        </is>
-      </c>
-      <c r="F1" s="72" t="inlineStr">
-        <is>
-          <t>Ticket/ Bug ID</t>
-        </is>
-      </c>
-      <c r="G1" s="72" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
-      </c>
-      <c r="H1" s="101" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="162" t="inlineStr">
-        <is>
-          <t>Case List Map</t>
-        </is>
-      </c>
-      <c r="B2" s="150" t="n"/>
-      <c r="C2" s="150" t="n"/>
-      <c r="D2" s="150" t="n"/>
-      <c r="E2" s="150" t="n"/>
-      <c r="F2" s="150" t="n"/>
-      <c r="G2" s="151" t="n"/>
-      <c r="H2" s="66" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="96" t="inlineStr">
-        <is>
-          <t>Map_01</t>
-        </is>
-      </c>
-      <c r="B3" s="97" t="inlineStr">
-        <is>
-          <t>Verify user is able to configure geo options</t>
-        </is>
-      </c>
-      <c r="C3" s="97" t="inlineStr">
-        <is>
-          <t>1. Login to CC HQ
-2. Navigate to applications 
-3. select any case list application
-4. Navigate to case list settings 
-5. Go to case list tab
-6. Under display properties configure the geo boundary and geo points'
-Note: Geo boundary and geo points options are visible only when address property is configured</t>
-        </is>
-      </c>
-      <c r="D3" s="97" t="inlineStr">
-        <is>
-          <t>- Geo boundary and geopoints options are available only when address display property is added
-- Geo boundary colour is available when geo boundary options is configured
-- Geo points colour is available when geo points option is configured
-- When "Address" property is deleted , Geo boundary and geo points options are automatically removed and  "requires column with format: Address" message is dispalyed
- - When geo boundary is deleted, geo boundary colour is automatically removed and message is displayed
-- When geo point is deleted, geo point colour is automatically removed and message is displayed</t>
-        </is>
-      </c>
-      <c r="E3" s="66" t="n"/>
-      <c r="F3" s="66" t="n"/>
-      <c r="G3" s="66" t="n"/>
-      <c r="H3" s="103" t="inlineStr">
-        <is>
-          <t>Refer these tests to configure case list map properties - https://docs.google.com/spreadsheets/d/1ENauf0cWqR0c9Seu29xarLucB78j3bNJzuQ7ut0T7Fs/edit?gid=2#gid=2&amp;range=18:23</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="96" t="inlineStr">
-        <is>
-          <t>Map_02</t>
-        </is>
-      </c>
-      <c r="B4" s="104" t="inlineStr">
-        <is>
-          <t>Verify removal of required Geo options</t>
-        </is>
-      </c>
-      <c r="C4" s="97" t="inlineStr">
-        <is>
-          <t>Continue to above TC:
- - Remove address property, check informational message is displayed
- Repeated the above step with geo boundary and geo points</t>
-        </is>
-      </c>
-      <c r="D4" s="97" t="inlineStr">
-        <is>
-          <t>- When "Address" property is deleted , Geo boundary and geo points options are automatically removed and  "requires column with format: Address" message is dispalyed
- - When geo boundary is deleted, geo boundary colour is automatically removed and message is displayed
-- When geo point is deleted, geo point colour is automatically removed and message is displayed</t>
-        </is>
-      </c>
-      <c r="E4" s="66" t="n"/>
-      <c r="F4" s="66" t="n"/>
-      <c r="G4" s="66" t="n"/>
-      <c r="H4" s="66" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="96" t="inlineStr">
-        <is>
-          <t>Map_03</t>
-        </is>
-      </c>
-      <c r="B5" s="97" t="inlineStr">
-        <is>
-          <t>Verify polygons and points are displayed on the case list map</t>
-        </is>
-      </c>
-      <c r="C5" s="97" t="inlineStr">
-        <is>
-          <t>1. Install CCC app
-2. Install the app used in map_01
-3. Login to the app
-4. Submit few forms with boundary box and points data and colours in hex code
-5. Navigate to case list follow up form
-6. Click on three dots menu
-7. Click on view map</t>
-        </is>
-      </c>
-      <c r="D5" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">- Polygons as per submitted data and colors should get highligted on the map
-</t>
-        </is>
-      </c>
-      <c r="E5" s="66" t="n"/>
-      <c r="F5" s="66" t="n"/>
-      <c r="G5" s="66" t="n"/>
-      <c r="H5" s="66" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="96" t="inlineStr">
-        <is>
-          <t>Map_04</t>
-        </is>
-      </c>
-      <c r="B6" s="104" t="inlineStr">
-        <is>
-          <t>Verify multiple locations display correctly</t>
-        </is>
-      </c>
-      <c r="C6" s="97" t="inlineStr">
-        <is>
-          <t>1. Submit multiple forms with different locations
-2. Navigate to case list
-3. Click on 3 dots menu &gt;&gt; view on map</t>
-        </is>
-      </c>
-      <c r="D6" s="97" t="inlineStr">
-        <is>
-          <t>- Multiple polygonas and points are visible clearly on the map with their resspective submitted colors</t>
-        </is>
-      </c>
-      <c r="E6" s="66" t="n"/>
-      <c r="F6" s="66" t="n"/>
-      <c r="G6" s="66" t="n"/>
-      <c r="H6" s="66" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="96" t="inlineStr">
-        <is>
-          <t>Map_05</t>
-        </is>
-      </c>
-      <c r="B7" s="104" t="inlineStr">
-        <is>
-          <t>Verify overlapping polygons for same coordinates</t>
-        </is>
-      </c>
-      <c r="C7" s="97" t="inlineStr">
-        <is>
-          <t>1. Submit the 2 or 3 forms with same boundary and points details
-2.  Navigate to case list
-3. Click on 3 dots menu &gt;&gt; view on map</t>
-        </is>
-      </c>
-      <c r="D7" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">- Cases with same location get overlap on each other and only one case is highlighted </t>
-        </is>
-      </c>
-      <c r="E7" s="66" t="n"/>
-      <c r="F7" s="66" t="n"/>
-      <c r="G7" s="66" t="n"/>
-      <c r="H7" s="66" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="96" t="inlineStr">
-        <is>
-          <t>Map_06</t>
-        </is>
-      </c>
-      <c r="B8" s="104" t="inlineStr">
-        <is>
-          <t>Verify case name popup appears on clicking a polygon</t>
-        </is>
-      </c>
-      <c r="C8" s="105" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
-Click on a polygon on the map.</t>
-        </is>
-      </c>
-      <c r="D8" s="97" t="inlineStr">
-        <is>
-          <t>- Case name appears upon clicking on the polygon</t>
-        </is>
-      </c>
-      <c r="E8" s="66" t="n"/>
-      <c r="F8" s="66" t="n"/>
-      <c r="G8" s="66" t="n"/>
-      <c r="H8" s="66" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="96" t="inlineStr">
-        <is>
-          <t>Map_07</t>
-        </is>
-      </c>
-      <c r="B9" s="104" t="inlineStr">
-        <is>
-          <t>Verify user can open the Case Follow-Up form by clicking on case name</t>
-        </is>
-      </c>
-      <c r="C9" s="97" t="inlineStr">
-        <is>
-          <t>Click on the case name on the map</t>
-        </is>
-      </c>
-      <c r="D9" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> - User redirects to the case follow up form</t>
-        </is>
-      </c>
-      <c r="E9" s="66" t="n"/>
-      <c r="F9" s="66" t="n"/>
-      <c r="G9" s="66" t="n"/>
-      <c r="H9" s="66" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="96" t="inlineStr">
-        <is>
-          <t>Map_08</t>
-        </is>
-      </c>
-      <c r="B10" s="104" t="inlineStr">
-        <is>
-          <t>Verify warning message on the mobile map for wrong configuration</t>
-        </is>
-      </c>
-      <c r="C10" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. Submit few forms with geo boundary and point details
-2. Few forms with out complete or incorrect details
-3. Navigate to case list form &gt;&gt; view on map
-</t>
-        </is>
-      </c>
-      <c r="D10" s="97" t="inlineStr">
-        <is>
-          <t>- User should see a below message at the bottom of screen 
-"There was an error in app configuration due to which not all markers on the map are loaded correctly.”</t>
-        </is>
-      </c>
-      <c r="E10" s="66" t="n"/>
-      <c r="F10" s="66" t="n"/>
-      <c r="G10" s="66" t="n"/>
-      <c r="H10" s="66" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="96" t="inlineStr">
-        <is>
-          <t>Map_09</t>
-        </is>
-      </c>
-      <c r="B11" s="104" t="inlineStr">
-        <is>
-          <t>Verify visibility of individual toggles based on entity count</t>
-        </is>
-      </c>
-      <c r="C11" s="97" t="inlineStr">
-        <is>
-          <t>1. Submit only one form with one entity either boundary box or points
-2. Navigate to case list map</t>
-        </is>
-      </c>
-      <c r="D11" s="97" t="inlineStr">
-        <is>
-          <t>- Toggle buttons are not visible and by default they are in "ON"
--  toggle panel is hidden if less than two toggles are needed
-- Location should get highlighted as per your form submission</t>
-        </is>
-      </c>
-      <c r="E11" s="66" t="n"/>
-      <c r="F11" s="66" t="n"/>
-      <c r="G11" s="66" t="n"/>
-      <c r="H11" s="66" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="96" t="inlineStr">
-        <is>
-          <t>Map_10</t>
-        </is>
-      </c>
-      <c r="B12" s="104" t="inlineStr">
-        <is>
-          <t>Verify toggles are shown when multiple entities exist</t>
-        </is>
-      </c>
-      <c r="C12" s="97" t="inlineStr">
-        <is>
-          <t>1. Submit multiple forms with multiple entities
-2. Navigate to case list map</t>
-        </is>
-      </c>
-      <c r="D12" s="97" t="inlineStr">
-        <is>
-          <t>- Toggle buttons are visible
-- Entire toggle panel is shown if at least two toggles are needed</t>
-        </is>
-      </c>
-      <c r="E12" s="66" t="n"/>
-      <c r="F12" s="66" t="n"/>
-      <c r="G12" s="66" t="n"/>
-      <c r="H12" s="66" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="96" t="inlineStr">
-        <is>
-          <t>Map_11</t>
-        </is>
-      </c>
-      <c r="B13" s="104" t="inlineStr">
-        <is>
-          <t>Verify user can toggle polygons and points ON/OFF</t>
-        </is>
-      </c>
-      <c r="C13" s="97" t="inlineStr">
-        <is>
-          <t>continue to above TC:
- - Toggle off the polygons button, ON the geo points
- - Toggle off the geopoints button, On the polygons button
- - Off both at a time</t>
-        </is>
-      </c>
-      <c r="D13" s="97" t="inlineStr">
-        <is>
-          <t>- By default polygons and geo points are ON
-- When user off the polyongs, boundary colour is not shown and only point is shown on map
-- When user off the geopoints, boundary is shown and point is not shown
-- When turn off both , neither points nor boundary are visible</t>
-        </is>
-      </c>
-      <c r="E13" s="66" t="n"/>
-      <c r="F13" s="66" t="n"/>
-      <c r="G13" s="66" t="n"/>
-      <c r="H13" s="66" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:G2"/>
-  </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="E3:E13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Pass,Fail,N/A,Blocking"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" location="gid=2&amp;range=18:23" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Expand Legend into a full Read Me / Tab Guide
Paragraph briefs for every tab (what each refers to), the two-outputs framing,
the one-line Gap-Analysis-vs-Automation-Coverage distinction, plus the row-type /
Bucket / Eng Coverage / Action definitions. Renamed tab Legend -> Read Me.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Legend" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name=" Test Tracker" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Personal ID Tests" sheetId="4" state="visible" r:id="rId4"/>
@@ -28,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="27">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -154,6 +154,14 @@
     <font>
       <b val="1"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
     </font>
   </fonts>
   <fills count="20">
@@ -403,7 +411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="171">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -851,6 +859,12 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1277,222 +1291,434 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" style="145" min="1" max="1"/>
-    <col width="95" customWidth="1" style="145" min="2" max="2"/>
+    <col width="42" customWidth="1" style="145" min="1" max="1"/>
+    <col width="100" customWidth="1" style="145" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="167" t="inlineStr">
-        <is>
-          <t>Connect QA Gap Analysis — Legend</t>
-        </is>
-      </c>
-      <c r="B1" s="166" t="inlineStr"/>
+      <c r="A1" s="171" t="inlineStr">
+        <is>
+          <t>Read Me — Tab Guide &amp; Legend</t>
+        </is>
+      </c>
+      <c r="B1" s="166" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="166" t="inlineStr"/>
-      <c r="B2" s="166" t="inlineStr"/>
+      <c r="A2" s="172" t="inlineStr">
+        <is>
+          <t>Connect QA Gap Analysis · Mobile App Regression stream</t>
+        </is>
+      </c>
+      <c r="B2" s="166" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="168" t="inlineStr">
-        <is>
-          <t>ROW TYPES (Gap Analysis tab) — identified by the Gap ID prefix</t>
-        </is>
-      </c>
-      <c r="B3" s="166" t="inlineStr"/>
+      <c r="A3" s="166" t="inlineStr"/>
+      <c r="B3" s="166" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="166" t="inlineStr">
-        <is>
-          <t>Functional gap</t>
-        </is>
-      </c>
-      <c r="B4" s="166" t="inlineStr">
-        <is>
-          <t>Product behaviour that exists in the code but has NO test case in this MTP. The core deliverable; candidates for QA test coverage. IDs: GAP-SRC-*, GAP-BE-*, GAP-FE-*.</t>
-        </is>
-      </c>
+      <c r="A4" s="168" t="inlineStr">
+        <is>
+          <t>WHAT THIS EXERCISE PRODUCED — two separate outputs</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="166" t="inlineStr">
         <is>
-          <t>Unit-test-coverage gap (dev)</t>
+          <t>Output 1: MTP completeness</t>
         </is>
       </c>
       <c r="B5" s="166" t="inlineStr">
         <is>
-          <t>Where the ENGINEERING product code lacks a unit test. A note for the dev teams (not QA automation). IDs: GAP-UTC-*.</t>
+          <t>Everything the product does that was NOT documented in this test plan. ALL functional gaps get added to the plan, whether or not engineering already tests them.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="166" t="inlineStr">
         <is>
-          <t>Cross-cutting</t>
+          <t>Output 2: QA automation backlog</t>
         </is>
       </c>
       <c r="B6" s="166" t="inlineStr">
         <is>
-          <t>Not a single missing case: hygiene (e.g. duplicate IDs), MTP-vs-code discrepancies, or automation/dead-code notes. Fix-the-plan / fix-the-code items. IDs: GAP-MISC-*, GAP-MMISC-*.</t>
+          <t>The subset of those gaps that QA still needs to automate — i.e. the ones engineering does NOT already cover. Filter the Action column for "Automate".</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="166" t="inlineStr"/>
-      <c r="B7" s="166" t="inlineStr"/>
+      <c r="B7" s="166" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="168" t="inlineStr">
         <is>
-          <t>BUCKET column</t>
-        </is>
-      </c>
-      <c r="B8" s="166" t="inlineStr"/>
+          <t>TAB GUIDE — what each tab is</t>
+        </is>
+      </c>
+      <c r="B8" s="166" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="166" t="inlineStr">
         <is>
-          <t>🟢 Already automated</t>
+          <t>Read Me</t>
         </is>
       </c>
       <c r="B9" s="166" t="inlineStr">
         <is>
-          <t>A spec exists and runs (tracked in the Automation Status tab, not here).</t>
+          <t>This tab. The key to the whole workbook.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="166" t="inlineStr">
         <is>
-          <t>🟡 Automatable - not yet done</t>
+          <t>Summary</t>
         </is>
       </c>
       <c r="B10" s="166" t="inlineStr">
         <is>
-          <t>Can be automated; this is the automation backlog.</t>
+          <t>A one-screen dashboard of the numbers, auto-calculated. Shows Output 1 (MTP completeness), Output 2 (automation backlog), plus dev unit-test and reconcile counts. Read this first for the big picture.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="166" t="inlineStr">
         <is>
-          <t>🔴 Manual only</t>
+          <t>Test Tracker / Test Tracker Horizontal</t>
         </is>
       </c>
       <c r="B11" s="166" t="inlineStr">
         <is>
-          <t>Impractical/impossible to automate (real SMS/OTP, push, camera, biometric, device, time-dependent).</t>
+          <t>ORIGINAL tabs (not from this exercise). The pre-existing execution trackers — who ran the manual test rounds and pass/fail counts. Left untouched.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="166" t="inlineStr"/>
-      <c r="B12" s="166" t="inlineStr"/>
+      <c r="A12" s="166" t="inlineStr">
+        <is>
+          <t>The surface tabs (Login, Opportunity creation, Visit verification, Microplanning, etc.)</t>
+        </is>
+      </c>
+      <c r="B12" s="166" t="inlineStr">
+        <is>
+          <t>ORIGINAL tabs. This IS the existing master test plan — the documented test cases grouped by product screen/area. The "before" picture that the gap analysis was measured against.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="168" t="inlineStr">
-        <is>
-          <t>ENG COVERAGE column (does engineering already test this, so QA avoids duplicating?)</t>
-        </is>
-      </c>
-      <c r="B13" s="166" t="inlineStr"/>
+      <c r="A13" s="166" t="inlineStr">
+        <is>
+          <t>Gap Analysis  (MAIN OUTPUT)</t>
+        </is>
+      </c>
+      <c r="B13" s="166" t="inlineStr">
+        <is>
+          <t>Every coverage gap we found — behaviour that exists in the product code but had NO case in the surface tabs. Each row carries its Bucket, Eng Coverage, and Action. This is the deliverable: what was missing, and what to do about it. Reviewers work here.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="166" t="inlineStr">
         <is>
-          <t>Eng-covered (logic)</t>
+          <t>Automation Coverage</t>
         </is>
       </c>
       <c r="B14" s="166" t="inlineStr">
         <is>
-          <t>Eng PR-run tests cover the logic. QA adds an e2e test only if on a critical user journey.</t>
+          <t>The pass-1 baseline: the existing master test cases checked against QA's CURRENT automated suite (the pytest tests in dimagi-qa-ccc) — "of what we already documented, how much is automated." Migration bookkeeping; context, not the headline.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="166" t="inlineStr">
         <is>
-          <t>QA-owned</t>
+          <t>Automation Status</t>
         </is>
       </c>
       <c r="B15" s="166" t="inlineStr">
         <is>
-          <t>Real device/external (SMS/OTP/push/camera) — eng cannot unit-test either. QA-owned priority.</t>
+          <t>The short list of master-plan cases confirmed as ALREADY automated (the green cases). "What is already done."</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="166" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="B16" s="166" t="inlineStr">
-        <is>
-          <t>Some eng coverage; confirm with eng.</t>
-        </is>
-      </c>
+      <c r="A16" s="166" t="inlineStr"/>
+      <c r="B16" s="166" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="166" t="inlineStr">
         <is>
-          <t>Eng GAP</t>
-        </is>
-      </c>
-      <c r="B17" s="166" t="inlineStr">
-        <is>
-          <t>Eng has no unit test here (a GAP-UTC row).</t>
-        </is>
-      </c>
+          <t>ONE-LINE DISTINCTION</t>
+        </is>
+      </c>
+      <c r="B17" s="166" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="166" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="A18" s="168" t="inlineStr">
+        <is>
+          <t>Gap Analysis</t>
         </is>
       </c>
       <c r="B18" s="166" t="inlineStr">
         <is>
-          <t>Hygiene/discrepancy/automation note.</t>
+          <t>What was MISSING from the plan (new findings from reading the code) = completeness of the plan.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="166" t="inlineStr"/>
-      <c r="B19" s="166" t="inlineStr"/>
+      <c r="A19" s="166" t="inlineStr">
+        <is>
+          <t>Automation Coverage / Status</t>
+        </is>
+      </c>
+      <c r="B19" s="166" t="inlineStr">
+        <is>
+          <t>Of what was ALREADY in the plan, how much is automated = automation of the plan.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="168" t="inlineStr">
-        <is>
-          <t>OTHER TABS</t>
-        </is>
-      </c>
-      <c r="B20" s="166" t="inlineStr"/>
+      <c r="A20" s="166" t="inlineStr"/>
+      <c r="B20" s="166" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="166" t="inlineStr">
-        <is>
-          <t>Automation Coverage</t>
-        </is>
-      </c>
-      <c r="B21" s="166" t="inlineStr">
-        <is>
-          <t>Pass-1 baseline: MTP cases vs the existing QA automated suite (migration input, not this exercise's headline).</t>
-        </is>
-      </c>
+      <c r="A21" s="168" t="inlineStr">
+        <is>
+          <t>GAP ANALYSIS — the 3 row types (by Gap ID prefix)</t>
+        </is>
+      </c>
+      <c r="B21" s="166" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="166" t="inlineStr">
         <is>
-          <t>Automation Status</t>
+          <t>Functional gap</t>
         </is>
       </c>
       <c r="B22" s="166" t="inlineStr">
         <is>
-          <t>MTP cases confirmed already automated (green).</t>
+          <t>Behaviour in the code with no test case in the MTP. The core finding; QA-automation candidates. IDs: GAP-SRC-*, GAP-BE-*, GAP-FE-*.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="166" t="inlineStr">
+        <is>
+          <t>Unit-test-coverage gap (dev)</t>
+        </is>
+      </c>
+      <c r="B23" s="166" t="inlineStr">
+        <is>
+          <t>Where the ENGINEERING code lacks a unit test. A note for dev teams, not QA automation. IDs: GAP-UTC-*.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="166" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="B24" s="166" t="inlineStr">
+        <is>
+          <t>Not a single missing case: hygiene (e.g. duplicate IDs), MTP-vs-code discrepancies, or automation/dead-code notes. IDs: GAP-MISC-*, GAP-MMISC-*.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="166" t="inlineStr"/>
+      <c r="B25" s="166" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="166" t="inlineStr">
+        <is>
+          <t>BUCKET column</t>
+        </is>
+      </c>
+      <c r="B26" s="166" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="168" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="B27" s="166" t="inlineStr">
+        <is>
+          <t>A spec exists and runs (tracked in Automation Status).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="166" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="B28" s="166" t="inlineStr">
+        <is>
+          <t>Can be automated; the automation backlog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="166" t="inlineStr">
+        <is>
+          <t>🔴 Manual only</t>
+        </is>
+      </c>
+      <c r="B29" s="166" t="inlineStr">
+        <is>
+          <t>Impractical/impossible to automate (real SMS/OTP, push, camera, biometric, device, time-dependent).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="166" t="inlineStr"/>
+      <c r="B30" s="166" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="166" t="inlineStr">
+        <is>
+          <t>ENG COVERAGE column — does engineering already test this? (avoid duplicating eng work)</t>
+        </is>
+      </c>
+      <c r="B31" s="166" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="168" t="inlineStr">
+        <is>
+          <t>Eng-covered (logic)</t>
+        </is>
+      </c>
+      <c r="B32" s="166" t="inlineStr">
+        <is>
+          <t>Eng PR-run tests cover the logic. QA adds an e2e test only if on a critical user journey.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned</t>
+        </is>
+      </c>
+      <c r="B33" s="166" t="inlineStr">
+        <is>
+          <t>Real device/external (SMS/OTP/push/camera) — eng cannot unit-test either. QA-owned priority.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="166" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="B34" s="166" t="inlineStr">
+        <is>
+          <t>Some eng coverage; confirm with eng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="166" t="inlineStr">
+        <is>
+          <t>Eng GAP</t>
+        </is>
+      </c>
+      <c r="B35" s="166" t="inlineStr">
+        <is>
+          <t>Eng has no unit test here (a GAP-UTC row).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="166" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B36" s="166" t="inlineStr">
+        <is>
+          <t>Hygiene/discrepancy/automation note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="166" t="inlineStr"/>
+      <c r="B37" s="166" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="166" t="inlineStr">
+        <is>
+          <t>ACTION column — the decision per row</t>
+        </is>
+      </c>
+      <c r="B38" s="166" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="168" t="inlineStr">
+        <is>
+          <t>Add to MTP only (eng-covered)</t>
+        </is>
+      </c>
+      <c r="B39" s="166" t="inlineStr">
+        <is>
+          <t>Document it in the plan; do NOT automate — eng already tests it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (QA-owned)</t>
+        </is>
+      </c>
+      <c r="B40" s="166" t="inlineStr">
+        <is>
+          <t>Add to plan AND automate — eng cannot cover it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="166" t="inlineStr">
+        <is>
+          <t>Add to MTP + Automate (confirm w/ eng)</t>
+        </is>
+      </c>
+      <c r="B41" s="166" t="inlineStr">
+        <is>
+          <t>Add to plan; likely automate — confirm eng coverage first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="166" t="inlineStr">
+        <is>
+          <t>Dev: add unit test</t>
+        </is>
+      </c>
+      <c r="B42" s="166" t="inlineStr">
+        <is>
+          <t>For the dev team — product code missing a unit test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="166" t="inlineStr">
+        <is>
+          <t>Reconcile (plan/code)</t>
+        </is>
+      </c>
+      <c r="B43" s="166" t="inlineStr">
+        <is>
+          <t>Fix the plan or the code (hygiene / discrepancy).</t>
         </is>
       </c>
     </row>
@@ -19534,7 +19760,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="0" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="170" t="inlineStr">
@@ -19542,35 +19768,35 @@
           <t>OUTPUT 1 — MTP completeness (all functional gaps: add to the MTP)</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" s="0">
         <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"Add to MTP*")</f>
         <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">   ...of which already eng-covered (add to MTP only, do NOT automate)</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B4" s="0">
         <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"Add to MTP only*")</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">   ...of which QA to automate (see Output 2)</t>
         </is>
       </c>
-      <c r="B5">
+      <c r="B5" s="0">
         <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"*Automate*")</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" s="0" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="170" t="inlineStr">
@@ -19578,35 +19804,35 @@
           <t>OUTPUT 2 — QA automation backlog (functional gaps NOT eng-covered)</t>
         </is>
       </c>
-      <c r="B7">
+      <c r="B7" s="0">
         <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"*Automate*")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">   QA-owned (real device/SMS/push - eng cannot cover)</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B8" s="0">
         <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"*QA-owned*")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">   Automatable, confirm w/ eng (partial coverage)</t>
         </is>
       </c>
-      <c r="B9">
+      <c r="B9" s="0">
         <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"*confirm w/ eng*")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" s="0" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="170" t="inlineStr">
@@ -19614,7 +19840,7 @@
           <t>DEV deliverable — unit-test-coverage gaps (eng to add unit tests)</t>
         </is>
       </c>
-      <c r="B11">
+      <c r="B11" s="0">
         <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"Dev:*")</f>
         <v/>
       </c>
@@ -19625,13 +19851,13 @@
           <t>CROSS-CUTTING — reconcile plan/code (hygiene/discrepancy)</t>
         </is>
       </c>
-      <c r="B12">
+      <c r="B12" s="0">
         <f>COUNTIF('Gap Analysis'!$L$2:$L$1000,"Reconcile*")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" s="0" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="170" t="inlineStr">
@@ -19639,7 +19865,7 @@
           <t>TOTAL Gap Analysis rows</t>
         </is>
       </c>
-      <c r="B14">
+      <c r="B14" s="0">
         <f>COUNTA('Gap Analysis'!$L$2:$L$1000)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add live Coverage Tracker tab (playbook pattern, as done for SureAdhere)
Per-surface automation coverage of existing MTP cases (Automated/Automatable-not-
built/Manual/Total/% Automated) via COUNTIF/COUNTIFS against Automation Status +
Automation Coverage, with a TOTAL row, plus a Gap Analysis rollup of the new
findings. Left the original manual-execution Test Tracker tabs untouched (they use
Google-Sheets-only sheetName() formulas). Web 9% automated (28/316), Mobile 20%
(34/166).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -5,18 +5,19 @@
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name=" Test Tracker" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Personal ID Tests" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Integration Tests (Connect)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Connect Landing Page" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Connect messaging" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Connect Notifications" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Connect worker History" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Case List map " sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Test Tracker Horizontal" sheetId="11" state="hidden" r:id="rId11"/>
-    <sheet name="Automation Status" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Gap Analysis" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Automation Coverage" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Coverage Tracker" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name=" Test Tracker" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Personal ID Tests" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Integration Tests (Connect)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Connect Landing Page" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Connect messaging" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Connect Notifications" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Connect worker History" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Case List map " sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Test Tracker Horizontal" sheetId="12" state="hidden" r:id="rId12"/>
+    <sheet name="Automation Status" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Gap Analysis" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Automation Coverage" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="29">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -163,8 +164,15 @@
       <i val="1"/>
       <color rgb="00555555"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -276,6 +284,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -411,7 +429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="180">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -865,6 +883,27 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="23" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1733,6 +1772,173 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="19" customWidth="1" style="145" min="1" max="1"/>
+    <col width="37.75" customWidth="1" style="145" min="2" max="2"/>
+    <col width="44.63" customWidth="1" style="145" min="3" max="3"/>
+    <col width="39.88" customWidth="1" style="145" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="72" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B1" s="72" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steps </t>
+        </is>
+      </c>
+      <c r="D1" s="72" t="inlineStr">
+        <is>
+          <t>Expected Outcome</t>
+        </is>
+      </c>
+      <c r="E1" s="72" t="inlineStr">
+        <is>
+          <t>Status (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="F1" s="72" t="inlineStr">
+        <is>
+          <t>Ticket/ Bug ID</t>
+        </is>
+      </c>
+      <c r="G1" s="72" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="H1" s="72" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="96" t="inlineStr">
+        <is>
+          <t>Worker_History 1</t>
+        </is>
+      </c>
+      <c r="B2" s="97" t="inlineStr">
+        <is>
+          <t>Verify we are able create manage creditals on CCC web UI</t>
+        </is>
+      </c>
+      <c r="C2" s="97" t="inlineStr">
+        <is>
+          <t>1. Login CCC web UI
+2. Navigte to opportunity dashboard
+3. Click on hamburger option
+4. Select edit opportunity
+5. Verify manage credentials section is visible
+6.Click on Learn Level field, the following options contains in the dropdown:
+    - None
+    - Learning passed 
+7. Click on Delivery level field, the dropdown contains following options:
+    - None
+    - 25 deliveries
+    - 50 deliveries
+    - 100 deliveries
+    - 200 deliveries
+    - 500 deliveries
+    - 1000 deliveries
+8. Select any option [except none - it is for disable] from learn level and  delivery level fields 
+9. Click submit</t>
+        </is>
+      </c>
+      <c r="D2" s="97" t="inlineStr">
+        <is>
+          <t>- User should be able to add credentials succesfully</t>
+        </is>
+      </c>
+      <c r="E2" s="100" t="n"/>
+      <c r="F2" s="66" t="n"/>
+      <c r="G2" s="66" t="n"/>
+      <c r="H2" s="66" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="96" t="inlineStr">
+        <is>
+          <t>Worker_History 2</t>
+        </is>
+      </c>
+      <c r="B3" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify earned credentials are visible in worker history section </t>
+        </is>
+      </c>
+      <c r="C3" s="97" t="inlineStr">
+        <is>
+          <t>1. Sign up for personal ID [Mobile]
+2. Login to learn/delivery app
+3. Submit forms till reaches the credentials requirements
+4. Expand left hand menu &gt;&gt; select worker history page</t>
+        </is>
+      </c>
+      <c r="D3" s="97" t="inlineStr">
+        <is>
+          <t>- When user reaches the credentials requirement, they should earn the credential badges
+- Earned badges should be displayed on worker history page</t>
+        </is>
+      </c>
+      <c r="E3" s="66" t="n"/>
+      <c r="F3" s="66" t="n"/>
+      <c r="G3" s="66" t="n"/>
+      <c r="H3" s="66" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="96" t="inlineStr">
+        <is>
+          <t>Worker_History 3</t>
+        </is>
+      </c>
+      <c r="B4" s="97" t="inlineStr">
+        <is>
+          <t>Verify previously earned credentials are still visible on mobile when disabled on web UI</t>
+        </is>
+      </c>
+      <c r="C4" s="97" t="inlineStr">
+        <is>
+          <t>1.Disable the credentials in web UI
+2. Navigate to worker history page in mobile
+3. Verify the previoulsy earned badges are still remain</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>-User should see the previously earned badges should be visible even after disabling the credentials on web UI</t>
+        </is>
+      </c>
+      <c r="E4" s="66" t="n"/>
+      <c r="F4" s="66" t="n"/>
+      <c r="G4" s="66" t="n"/>
+      <c r="H4" s="66" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="E2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,N/A,Blocking"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E3:E4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,N/A,Blocking"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
@@ -2147,7 +2353,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -7127,7 +7333,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8093,7 +8299,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13853,7 +14059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19876,6 +20082,430 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" style="145" min="1" max="1"/>
+    <col width="20" customWidth="1" style="145" min="2" max="2"/>
+    <col width="20" customWidth="1" style="145" min="3" max="3"/>
+    <col width="20" customWidth="1" style="145" min="4" max="4"/>
+    <col width="20" customWidth="1" style="145" min="5" max="5"/>
+    <col width="20" customWidth="1" style="145" min="6" max="6"/>
+    <col width="30" customWidth="1" style="145" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="173" t="inlineStr">
+        <is>
+          <t>Coverage Tracker — automation coverage of existing MTP cases (live)</t>
+        </is>
+      </c>
+      <c r="B1" s="166" t="n"/>
+      <c r="C1" s="166" t="n"/>
+      <c r="D1" s="166" t="n"/>
+      <c r="E1" s="166" t="n"/>
+      <c r="F1" s="166" t="n"/>
+      <c r="G1" s="166" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="166" t="n"/>
+      <c r="B2" s="166" t="n"/>
+      <c r="C2" s="166" t="n"/>
+      <c r="D2" s="166" t="n"/>
+      <c r="E2" s="166" t="n"/>
+      <c r="F2" s="166" t="n"/>
+      <c r="G2" s="166" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="168" t="inlineStr">
+        <is>
+          <t>Surface</t>
+        </is>
+      </c>
+      <c r="B3" s="168" t="inlineStr">
+        <is>
+          <t>Automated (built)</t>
+        </is>
+      </c>
+      <c r="C3" s="168" t="inlineStr">
+        <is>
+          <t>Automatable (not built)</t>
+        </is>
+      </c>
+      <c r="D3" s="168" t="inlineStr">
+        <is>
+          <t>Manual only</t>
+        </is>
+      </c>
+      <c r="E3" s="168" t="inlineStr">
+        <is>
+          <t>Total tracked</t>
+        </is>
+      </c>
+      <c r="F3" s="168" t="inlineStr">
+        <is>
+          <t>% Automated</t>
+        </is>
+      </c>
+      <c r="G3" s="168" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>Personal ID Tests</t>
+        </is>
+      </c>
+      <c r="B4" s="166">
+        <f>COUNTIF('Automation Status'!$A:$A,$A4)</f>
+        <v/>
+      </c>
+      <c r="C4" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A4,'Automation Coverage'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D4" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A4,'Automation Coverage'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E4" s="166">
+        <f>B4+C4+D4</f>
+        <v/>
+      </c>
+      <c r="F4" s="174">
+        <f>IF(E4&gt;0,B4/E4,0)</f>
+        <v/>
+      </c>
+      <c r="G4" s="166" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="166" t="inlineStr">
+        <is>
+          <t>Integration Tests (Connect)</t>
+        </is>
+      </c>
+      <c r="B5" s="166">
+        <f>COUNTIF('Automation Status'!$A:$A,$A5)</f>
+        <v/>
+      </c>
+      <c r="C5" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A5,'Automation Coverage'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D5" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A5,'Automation Coverage'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E5" s="166">
+        <f>B5+C5+D5</f>
+        <v/>
+      </c>
+      <c r="F5" s="174">
+        <f>IF(E5&gt;0,B5/E5,0)</f>
+        <v/>
+      </c>
+      <c r="G5" s="166" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="166" t="inlineStr">
+        <is>
+          <t>Connect Landing Page</t>
+        </is>
+      </c>
+      <c r="B6" s="166">
+        <f>COUNTIF('Automation Status'!$A:$A,$A6)</f>
+        <v/>
+      </c>
+      <c r="C6" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A6,'Automation Coverage'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D6" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A6,'Automation Coverage'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E6" s="166">
+        <f>B6+C6+D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="174">
+        <f>IF(E6&gt;0,B6/E6,0)</f>
+        <v/>
+      </c>
+      <c r="G6" s="166" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="166" t="inlineStr">
+        <is>
+          <t>Connect messaging</t>
+        </is>
+      </c>
+      <c r="B7" s="166">
+        <f>COUNTIF('Automation Status'!$A:$A,$A7)</f>
+        <v/>
+      </c>
+      <c r="C7" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A7,'Automation Coverage'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D7" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A7,'Automation Coverage'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E7" s="166">
+        <f>B7+C7+D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="174">
+        <f>IF(E7&gt;0,B7/E7,0)</f>
+        <v/>
+      </c>
+      <c r="G7" s="166" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="166" t="inlineStr">
+        <is>
+          <t>Connect Notifications</t>
+        </is>
+      </c>
+      <c r="B8" s="166">
+        <f>COUNTIF('Automation Status'!$A:$A,$A8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A8,'Automation Coverage'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D8" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A8,'Automation Coverage'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E8" s="166">
+        <f>B8+C8+D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="174">
+        <f>IF(E8&gt;0,B8/E8,0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="166" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="166" t="inlineStr">
+        <is>
+          <t>Connect worker History</t>
+        </is>
+      </c>
+      <c r="B9" s="166">
+        <f>COUNTIF('Automation Status'!$A:$A,$A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A9,'Automation Coverage'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D9" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A9,'Automation Coverage'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E9" s="166">
+        <f>B9+C9+D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="174">
+        <f>IF(E9&gt;0,B9/E9,0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="166" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Case List map </t>
+        </is>
+      </c>
+      <c r="B10" s="166">
+        <f>COUNTIF('Automation Status'!$A:$A,$A10)</f>
+        <v/>
+      </c>
+      <c r="C10" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A10,'Automation Coverage'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D10" s="166">
+        <f>COUNTIFS('Automation Coverage'!$B:$B,$A10,'Automation Coverage'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E10" s="166">
+        <f>B10+C10+D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="174">
+        <f>IF(E10&gt;0,B10/E10,0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="166" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="175" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="175">
+        <f>SUM(B4:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="175">
+        <f>SUM(C4:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="175">
+        <f>SUM(D4:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="175">
+        <f>SUM(E4:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="176">
+        <f>IF(E11&gt;0,B11/E11,0)</f>
+        <v/>
+      </c>
+      <c r="G11" s="175" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="166" t="n"/>
+      <c r="B12" s="166" t="n"/>
+      <c r="C12" s="166" t="n"/>
+      <c r="D12" s="166" t="n"/>
+      <c r="E12" s="166" t="n"/>
+      <c r="F12" s="166" t="n"/>
+      <c r="G12" s="166" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="177" t="inlineStr">
+        <is>
+          <t>Gap Analysis — new findings from source analysis (not in the counts above)</t>
+        </is>
+      </c>
+      <c r="B13" s="166" t="n"/>
+      <c r="C13" s="166" t="n"/>
+      <c r="D13" s="166" t="n"/>
+      <c r="E13" s="166" t="n"/>
+      <c r="F13" s="166" t="n"/>
+      <c r="G13" s="166" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="178" t="inlineStr">
+        <is>
+          <t>Output 1: functional gaps to ADD to MTP</t>
+        </is>
+      </c>
+      <c r="B14" s="166">
+        <f>COUNTIF('Gap Analysis'!$L:$L,"Add to MTP*")</f>
+        <v/>
+      </c>
+      <c r="C14" s="166" t="n"/>
+      <c r="D14" s="166" t="n"/>
+      <c r="E14" s="166" t="n"/>
+      <c r="F14" s="166" t="n"/>
+      <c r="G14" s="166" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ...of which eng-covered (add to MTP only, do NOT automate)</t>
+        </is>
+      </c>
+      <c r="B15" s="166">
+        <f>COUNTIF('Gap Analysis'!$L:$L,"Add to MTP only*")</f>
+        <v/>
+      </c>
+      <c r="C15" s="166" t="n"/>
+      <c r="D15" s="166" t="n"/>
+      <c r="E15" s="166" t="n"/>
+      <c r="F15" s="166" t="n"/>
+      <c r="G15" s="166" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="178" t="inlineStr">
+        <is>
+          <t>Output 2: functional gaps to AUTOMATE (QA backlog)</t>
+        </is>
+      </c>
+      <c r="B16" s="166">
+        <f>COUNTIF('Gap Analysis'!$L:$L,"*Automate*")</f>
+        <v/>
+      </c>
+      <c r="C16" s="166" t="n"/>
+      <c r="D16" s="166" t="n"/>
+      <c r="E16" s="166" t="n"/>
+      <c r="F16" s="166" t="n"/>
+      <c r="G16" s="166" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ...of which manual-only (red bucket)</t>
+        </is>
+      </c>
+      <c r="B17" s="166">
+        <f>COUNTIF('Gap Analysis'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="C17" s="166" t="n"/>
+      <c r="D17" s="166" t="n"/>
+      <c r="E17" s="166" t="n"/>
+      <c r="F17" s="166" t="n"/>
+      <c r="G17" s="166" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="178" t="inlineStr">
+        <is>
+          <t>Dev: unit-test-coverage gaps</t>
+        </is>
+      </c>
+      <c r="B18" s="166">
+        <f>COUNTIF('Gap Analysis'!$L:$L,"Dev:*")</f>
+        <v/>
+      </c>
+      <c r="C18" s="166" t="n"/>
+      <c r="D18" s="166" t="n"/>
+      <c r="E18" s="166" t="n"/>
+      <c r="F18" s="166" t="n"/>
+      <c r="G18" s="166" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="178" t="inlineStr">
+        <is>
+          <t>Cross-cutting: reconcile plan/code</t>
+        </is>
+      </c>
+      <c r="B19" s="166">
+        <f>COUNTIF('Gap Analysis'!$L:$L,"Reconcile*")</f>
+        <v/>
+      </c>
+      <c r="C19" s="166" t="n"/>
+      <c r="D19" s="166" t="n"/>
+      <c r="E19" s="166" t="n"/>
+      <c r="F19" s="166" t="n"/>
+      <c r="G19" s="166" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -20497,7 +21127,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFFFFFF"/>
@@ -21781,7 +22411,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -23446,7 +24076,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -24300,7 +24930,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -24702,7 +25332,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -25318,171 +25948,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="19" customWidth="1" style="145" min="1" max="1"/>
-    <col width="37.75" customWidth="1" style="145" min="2" max="2"/>
-    <col width="44.63" customWidth="1" style="145" min="3" max="3"/>
-    <col width="39.88" customWidth="1" style="145" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="72" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B1" s="72" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C1" s="72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Steps </t>
-        </is>
-      </c>
-      <c r="D1" s="72" t="inlineStr">
-        <is>
-          <t>Expected Outcome</t>
-        </is>
-      </c>
-      <c r="E1" s="72" t="inlineStr">
-        <is>
-          <t>Status (Pass/Fail)</t>
-        </is>
-      </c>
-      <c r="F1" s="72" t="inlineStr">
-        <is>
-          <t>Ticket/ Bug ID</t>
-        </is>
-      </c>
-      <c r="G1" s="72" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
-      </c>
-      <c r="H1" s="72" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="96" t="inlineStr">
-        <is>
-          <t>Worker_History 1</t>
-        </is>
-      </c>
-      <c r="B2" s="97" t="inlineStr">
-        <is>
-          <t>Verify we are able create manage creditals on CCC web UI</t>
-        </is>
-      </c>
-      <c r="C2" s="97" t="inlineStr">
-        <is>
-          <t>1. Login CCC web UI
-2. Navigte to opportunity dashboard
-3. Click on hamburger option
-4. Select edit opportunity
-5. Verify manage credentials section is visible
-6.Click on Learn Level field, the following options contains in the dropdown:
-    - None
-    - Learning passed 
-7. Click on Delivery level field, the dropdown contains following options:
-    - None
-    - 25 deliveries
-    - 50 deliveries
-    - 100 deliveries
-    - 200 deliveries
-    - 500 deliveries
-    - 1000 deliveries
-8. Select any option [except none - it is for disable] from learn level and  delivery level fields 
-9. Click submit</t>
-        </is>
-      </c>
-      <c r="D2" s="97" t="inlineStr">
-        <is>
-          <t>- User should be able to add credentials succesfully</t>
-        </is>
-      </c>
-      <c r="E2" s="100" t="n"/>
-      <c r="F2" s="66" t="n"/>
-      <c r="G2" s="66" t="n"/>
-      <c r="H2" s="66" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="96" t="inlineStr">
-        <is>
-          <t>Worker_History 2</t>
-        </is>
-      </c>
-      <c r="B3" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Verify earned credentials are visible in worker history section </t>
-        </is>
-      </c>
-      <c r="C3" s="97" t="inlineStr">
-        <is>
-          <t>1. Sign up for personal ID [Mobile]
-2. Login to learn/delivery app
-3. Submit forms till reaches the credentials requirements
-4. Expand left hand menu &gt;&gt; select worker history page</t>
-        </is>
-      </c>
-      <c r="D3" s="97" t="inlineStr">
-        <is>
-          <t>- When user reaches the credentials requirement, they should earn the credential badges
-- Earned badges should be displayed on worker history page</t>
-        </is>
-      </c>
-      <c r="E3" s="66" t="n"/>
-      <c r="F3" s="66" t="n"/>
-      <c r="G3" s="66" t="n"/>
-      <c r="H3" s="66" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="96" t="inlineStr">
-        <is>
-          <t>Worker_History 3</t>
-        </is>
-      </c>
-      <c r="B4" s="97" t="inlineStr">
-        <is>
-          <t>Verify previously earned credentials are still visible on mobile when disabled on web UI</t>
-        </is>
-      </c>
-      <c r="C4" s="97" t="inlineStr">
-        <is>
-          <t>1.Disable the credentials in web UI
-2. Navigate to worker history page in mobile
-3. Verify the previoulsy earned badges are still remain</t>
-        </is>
-      </c>
-      <c r="D4" s="97" t="inlineStr">
-        <is>
-          <t>-User should see the previously earned badges should be visible even after disabling the credentials on web UI</t>
-        </is>
-      </c>
-      <c r="E4" s="66" t="n"/>
-      <c r="F4" s="66" t="n"/>
-      <c r="G4" s="66" t="n"/>
-      <c r="H4" s="66" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="E2" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Pass,Fail,N/A,Blocking"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E3:E4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"Pass,Fail,N/A,Blocking"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Eng-coverage pass on EXISTING MTP automatable cases
Applied the eng-coverage cross-ref to the automatable-not-built (yellow) existing
cases in Automation (existing MTP): added an Eng Coverage column. Finding: the
existing backlog is overwhelmingly UI/e2e (QA-owned) - web 171 QA-owned vs 36
likely-eng-covered; mobile 78 vs 2. Unlike the new gaps (mostly eng-covered),
the existing automation backlog genuinely needs QA automation. Dashboard shows
the rollup. Heuristic/best-guess pending eng confirmation.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -427,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="180">
+  <cellXfs count="181">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -902,6 +902,7 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7767,7 +7768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" style="145" min="1" max="1"/>
@@ -8208,6 +8209,36 @@
         <v/>
       </c>
       <c r="G21" s="175" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="180" t="inlineStr">
+        <is>
+          <t>EXISTING automatable-not-built cases — do they need automating?</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - need automating)</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>COUNTIF('Automation (existing MTP)'!$G:$G,"QA-owned (UI*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="166" t="inlineStr">
+        <is>
+          <t>Likely already eng-covered (confirm - may NOT need automating)</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>COUNTIF('Automation (existing MTP)'!$G:$G,"Partial*")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13980,7 +14011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:G167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="145" min="1" max="1"/>
@@ -13989,6 +14020,7 @@
     <col width="26" customWidth="1" style="145" min="4" max="4"/>
     <col width="45" customWidth="1" style="145" min="5" max="5"/>
     <col width="26" customWidth="1" style="145" min="6" max="6"/>
+    <col width="44" customWidth="1" style="145" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14022,6 +14054,11 @@
           <t>Source</t>
         </is>
       </c>
+      <c r="G1" s="165" t="inlineStr">
+        <is>
+          <t>Eng Coverage</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="166" t="inlineStr">
@@ -14054,6 +14091,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G2" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="166" t="inlineStr">
@@ -14086,6 +14128,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G3" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="166" t="inlineStr">
@@ -14118,6 +14165,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="166" t="inlineStr">
@@ -14150,6 +14202,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G5" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="166" t="inlineStr">
@@ -14182,6 +14239,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G6" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="166" t="inlineStr">
@@ -14214,6 +14276,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G7" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="166" t="inlineStr">
@@ -14246,6 +14313,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G8" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="166" t="inlineStr">
@@ -14278,6 +14350,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G9" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="166" t="inlineStr">
@@ -14310,6 +14387,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G10" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="166" t="inlineStr">
@@ -14342,6 +14424,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G11" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="166" t="inlineStr">
@@ -14374,6 +14461,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G12" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="166" t="inlineStr">
@@ -14406,6 +14498,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G13" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="166" t="inlineStr">
@@ -14438,6 +14535,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G14" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="166" t="inlineStr">
@@ -14470,6 +14572,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G15" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="166" t="inlineStr">
@@ -14502,6 +14609,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G16" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="166" t="inlineStr">
@@ -14534,6 +14646,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G17" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="166" t="inlineStr">
@@ -14566,6 +14683,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G18" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="166" t="inlineStr">
@@ -14598,6 +14720,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G19" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="166" t="inlineStr">
@@ -14630,6 +14757,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G20" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="166" t="inlineStr">
@@ -14662,6 +14794,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G21" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="166" t="inlineStr">
@@ -14694,6 +14831,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G22" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="166" t="inlineStr">
@@ -14726,6 +14868,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G23" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="166" t="inlineStr">
@@ -14758,6 +14905,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G24" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="166" t="inlineStr">
@@ -14790,6 +14942,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G25" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="166" t="inlineStr">
@@ -14822,6 +14979,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G26" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="166" t="inlineStr">
@@ -14854,6 +15016,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G27" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="166" t="inlineStr">
@@ -14886,6 +15053,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G28" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="166" t="inlineStr">
@@ -14918,6 +15090,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G29" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="166" t="inlineStr">
@@ -14950,6 +15127,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G30" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="166" t="inlineStr">
@@ -14982,6 +15164,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G31" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="166" t="inlineStr">
@@ -15014,6 +15201,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G32" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="166" t="inlineStr">
@@ -15046,6 +15238,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G33" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="166" t="inlineStr">
@@ -15078,6 +15275,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G34" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="166" t="inlineStr">
@@ -15110,6 +15312,11 @@
           <t>Confirmed automated (pass 1)</t>
         </is>
       </c>
+      <c r="G35" s="166" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="166" t="inlineStr">
@@ -15142,6 +15349,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G36" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="166" t="inlineStr">
@@ -15174,6 +15386,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G37" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="166" t="inlineStr">
@@ -15206,6 +15423,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G38" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="166" t="inlineStr">
@@ -15238,6 +15460,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G39" s="166" t="inlineStr">
+        <is>
+          <t>Partial - likely eng-covered (confirm w/ eng)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="166" t="inlineStr">
@@ -15270,6 +15497,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G40" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="166" t="inlineStr">
@@ -15302,6 +15534,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G41" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="166" t="inlineStr">
@@ -15334,6 +15571,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G42" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="166" t="inlineStr">
@@ -15366,6 +15608,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G43" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="166" t="inlineStr">
@@ -15398,6 +15645,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G44" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="166" t="inlineStr">
@@ -15430,6 +15682,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G45" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="166" t="inlineStr">
@@ -15462,6 +15719,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G46" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="166" t="inlineStr">
@@ -15494,6 +15756,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G47" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="166" t="inlineStr">
@@ -15526,6 +15793,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G48" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="166" t="inlineStr">
@@ -15558,6 +15830,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G49" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="166" t="inlineStr">
@@ -15590,6 +15867,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G50" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="166" t="inlineStr">
@@ -15622,6 +15904,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G51" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="166" t="inlineStr">
@@ -15654,6 +15941,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G52" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="166" t="inlineStr">
@@ -15686,6 +15978,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G53" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="166" t="inlineStr">
@@ -15718,6 +16015,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G54" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="166" t="inlineStr">
@@ -15750,6 +16052,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G55" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="166" t="inlineStr">
@@ -15782,6 +16089,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G56" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="166" t="inlineStr">
@@ -15814,6 +16126,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G57" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="166" t="inlineStr">
@@ -15846,6 +16163,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G58" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="166" t="inlineStr">
@@ -15878,6 +16200,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G59" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="166" t="inlineStr">
@@ -15910,6 +16237,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G60" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="166" t="inlineStr">
@@ -15942,6 +16274,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G61" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="166" t="inlineStr">
@@ -15974,6 +16311,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G62" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="166" t="inlineStr">
@@ -16006,6 +16348,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G63" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="166" t="inlineStr">
@@ -16038,6 +16385,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G64" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="166" t="inlineStr">
@@ -16070,6 +16422,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G65" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="166" t="inlineStr">
@@ -16102,6 +16459,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G66" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="166" t="inlineStr">
@@ -16134,6 +16496,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G67" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="166" t="inlineStr">
@@ -16166,6 +16533,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G68" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="166" t="inlineStr">
@@ -16198,6 +16570,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G69" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="166" t="inlineStr">
@@ -16230,6 +16607,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G70" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="166" t="inlineStr">
@@ -16262,6 +16644,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G71" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="166" t="inlineStr">
@@ -16294,6 +16681,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G72" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="166" t="inlineStr">
@@ -16326,6 +16718,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G73" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="166" t="inlineStr">
@@ -16358,6 +16755,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G74" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="166" t="inlineStr">
@@ -16390,6 +16792,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G75" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="166" t="inlineStr">
@@ -16422,6 +16829,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G76" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="166" t="inlineStr">
@@ -16454,6 +16866,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G77" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="166" t="inlineStr">
@@ -16486,6 +16903,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G78" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="166" t="inlineStr">
@@ -16518,6 +16940,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G79" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="166" t="inlineStr">
@@ -16550,6 +16977,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G80" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="166" t="inlineStr">
@@ -16582,6 +17014,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G81" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="166" t="inlineStr">
@@ -16614,6 +17051,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G82" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="166" t="inlineStr">
@@ -16646,6 +17088,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G83" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="166" t="inlineStr">
@@ -16678,6 +17125,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G84" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="166" t="inlineStr">
@@ -16710,6 +17162,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G85" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="166" t="inlineStr">
@@ -16742,6 +17199,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G86" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="166" t="inlineStr">
@@ -16774,6 +17236,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G87" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="166" t="inlineStr">
@@ -16806,6 +17273,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G88" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="166" t="inlineStr">
@@ -16838,6 +17310,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G89" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="166" t="inlineStr">
@@ -16870,6 +17347,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G90" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="166" t="inlineStr">
@@ -16902,6 +17384,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G91" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="166" t="inlineStr">
@@ -16934,6 +17421,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G92" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="166" t="inlineStr">
@@ -16966,6 +17458,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G93" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="166" t="inlineStr">
@@ -16998,6 +17495,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G94" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="166" t="inlineStr">
@@ -17030,6 +17532,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G95" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="166" t="inlineStr">
@@ -17062,6 +17569,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G96" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="166" t="inlineStr">
@@ -17094,6 +17606,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G97" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="166" t="inlineStr">
@@ -17126,6 +17643,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G98" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="166" t="inlineStr">
@@ -17158,6 +17680,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G99" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="166" t="inlineStr">
@@ -17190,6 +17717,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G100" s="166" t="inlineStr">
+        <is>
+          <t>Partial - likely eng-covered (confirm w/ eng)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="166" t="inlineStr">
@@ -17222,6 +17754,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G101" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="166" t="inlineStr">
@@ -17254,6 +17791,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G102" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="166" t="inlineStr">
@@ -17286,6 +17828,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G103" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="166" t="inlineStr">
@@ -17318,6 +17865,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G104" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="166" t="inlineStr">
@@ -17350,6 +17902,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G105" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="166" t="inlineStr">
@@ -17382,6 +17939,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G106" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="166" t="inlineStr">
@@ -17414,6 +17976,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G107" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="166" t="inlineStr">
@@ -17446,6 +18013,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G108" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="166" t="inlineStr">
@@ -17478,6 +18050,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G109" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="166" t="inlineStr">
@@ -17510,6 +18087,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G110" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="166" t="inlineStr">
@@ -17542,6 +18124,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G111" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="166" t="inlineStr">
@@ -17574,6 +18161,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G112" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="166" t="inlineStr">
@@ -17606,6 +18198,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G113" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="166" t="inlineStr">
@@ -17638,6 +18235,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G114" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="166" t="inlineStr">
@@ -17670,6 +18272,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G115" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="166" t="inlineStr">
@@ -17702,6 +18309,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G116" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="166" t="inlineStr">
@@ -17734,6 +18346,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G117" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="166" t="inlineStr">
@@ -17766,6 +18383,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G118" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="166" t="inlineStr">
@@ -17798,6 +18420,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G119" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="166" t="inlineStr">
@@ -17830,6 +18457,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G120" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="166" t="inlineStr">
@@ -17862,6 +18494,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G121" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="166" t="inlineStr">
@@ -17894,6 +18531,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G122" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="166" t="inlineStr">
@@ -17926,6 +18568,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G123" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="166" t="inlineStr">
@@ -17958,6 +18605,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G124" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="166" t="inlineStr">
@@ -17990,6 +18642,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G125" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="166" t="inlineStr">
@@ -18022,6 +18679,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G126" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="166" t="inlineStr">
@@ -18054,6 +18716,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G127" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="166" t="inlineStr">
@@ -18086,6 +18753,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G128" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="166" t="inlineStr">
@@ -18118,6 +18790,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G129" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="166" t="inlineStr">
@@ -18150,6 +18827,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G130" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="166" t="inlineStr">
@@ -18182,6 +18864,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G131" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="166" t="inlineStr">
@@ -18214,6 +18901,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G132" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="166" t="inlineStr">
@@ -18246,6 +18938,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G133" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="166" t="inlineStr">
@@ -18278,6 +18975,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G134" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="166" t="inlineStr">
@@ -18310,6 +19012,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G135" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="166" t="inlineStr">
@@ -18342,6 +19049,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G136" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="166" t="inlineStr">
@@ -18374,6 +19086,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G137" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="166" t="inlineStr">
@@ -18406,6 +19123,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G138" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="166" t="inlineStr">
@@ -18438,6 +19160,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G139" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="166" t="inlineStr">
@@ -18470,6 +19197,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G140" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="166" t="inlineStr">
@@ -18502,6 +19234,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G141" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="166" t="inlineStr">
@@ -18534,6 +19271,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G142" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="166" t="inlineStr">
@@ -18566,6 +19308,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G143" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="166" t="inlineStr">
@@ -18598,6 +19345,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G144" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="166" t="inlineStr">
@@ -18630,6 +19382,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G145" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="166" t="inlineStr">
@@ -18662,6 +19419,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G146" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="166" t="inlineStr">
@@ -18694,6 +19456,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G147" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="166" t="inlineStr">
@@ -18726,6 +19493,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G148" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="166" t="inlineStr">
@@ -18758,6 +19530,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G149" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="166" t="inlineStr">
@@ -18790,6 +19567,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G150" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="166" t="inlineStr">
@@ -18822,6 +19604,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G151" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="166" t="inlineStr">
@@ -18854,6 +19641,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G152" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="166" t="inlineStr">
@@ -18886,6 +19678,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G153" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="166" t="inlineStr">
@@ -18918,6 +19715,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G154" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="166" t="inlineStr">
@@ -18950,6 +19752,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G155" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="166" t="inlineStr">
@@ -18982,6 +19789,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G156" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="166" t="inlineStr">
@@ -19014,6 +19826,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G157" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="166" t="inlineStr">
@@ -19046,6 +19863,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G158" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="166" t="inlineStr">
@@ -19078,6 +19900,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G159" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="166" t="inlineStr">
@@ -19110,6 +19937,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G160" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="166" t="inlineStr">
@@ -19142,6 +19974,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G161" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="166" t="inlineStr">
@@ -19174,6 +20011,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G162" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="166" t="inlineStr">
@@ -19206,6 +20048,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G163" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="166" t="inlineStr">
@@ -19238,6 +20085,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G164" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="166" t="inlineStr">
@@ -19270,6 +20122,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G165" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="166" t="inlineStr">
@@ -19302,6 +20159,11 @@
           <t>Pass 1 (mobile): MTP vs test suite</t>
         </is>
       </c>
+      <c r="G166" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="166" t="inlineStr">
@@ -19332,6 +20194,11 @@
       <c r="F167" s="166" t="inlineStr">
         <is>
           <t>Pass 1 (mobile): MTP vs test suite</t>
+        </is>
+      </c>
+      <c r="G167" s="166" t="inlineStr">
+        <is>
+          <t>QA-owned (manual)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Conclusions/Analysis Notes to Dashboard (reasoning travels with the sheet)
Prepended a 6-bullet Conclusions section to the Dashboard capturing the why:
method, the two outputs, new-gaps-mostly-eng-covered, existing-backlog-is-UI/e2e-
QA-owned, net savings on new gaps, and the best-guess caveat. Rebuilt the
Dashboard so Coverage Tracker formulas sit at correct row positions after the
insert (fixed a shifted-reference bug from the first attempt).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
+++ b/test_plans/CCC_Mobile_App_Regression_MTP.xlsx
@@ -170,7 +170,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -292,6 +292,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -427,7 +432,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="181">
+  <cellXfs count="183">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -903,6 +908,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7768,22 +7779,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="54" customWidth="1" style="145" min="1" max="1"/>
+    <col width="66" customWidth="1" style="145" min="1" max="1"/>
     <col width="20" customWidth="1" style="145" min="2" max="2"/>
     <col width="20" customWidth="1" style="145" min="3" max="3"/>
     <col width="20" customWidth="1" style="145" min="4" max="4"/>
     <col width="20" customWidth="1" style="145" min="5" max="5"/>
     <col width="20" customWidth="1" style="145" min="6" max="6"/>
-    <col width="28" customWidth="1" style="145" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="167" t="inlineStr">
         <is>
-          <t>Dashboard — outputs &amp; coverage (live)</t>
+          <t>Dashboard — conclusions, outputs &amp; coverage (live)</t>
         </is>
       </c>
       <c r="B1" s="166" t="n"/>
@@ -7791,454 +7801,526 @@
       <c r="D1" s="166" t="n"/>
       <c r="E1" s="166" t="n"/>
       <c r="F1" s="166" t="n"/>
-      <c r="G1" s="166" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="166" t="n"/>
+      <c r="A2" s="166" t="inlineStr"/>
       <c r="B2" s="166" t="n"/>
       <c r="C2" s="166" t="n"/>
       <c r="D2" s="166" t="n"/>
       <c r="E2" s="166" t="n"/>
       <c r="F2" s="166" t="n"/>
-      <c r="G2" s="166" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="177" t="inlineStr">
-        <is>
-          <t>OUTPUTS (from Gap Analysis)</t>
-        </is>
-      </c>
-      <c r="B3" s="166" t="inlineStr"/>
+      <c r="A3" s="182" t="inlineStr">
+        <is>
+          <t>CONCLUSIONS / ANALYSIS NOTES</t>
+        </is>
+      </c>
+      <c r="B3" s="166" t="n"/>
       <c r="C3" s="166" t="n"/>
       <c r="D3" s="166" t="n"/>
       <c r="E3" s="166" t="n"/>
       <c r="F3" s="166" t="n"/>
-      <c r="G3" s="166" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="166" t="inlineStr">
         <is>
-          <t>Output 1: functional gaps to ADD to MTP</t>
-        </is>
-      </c>
-      <c r="B4" s="166">
-        <f>COUNTIF('Gap Analysis'!$L:$L,"Add to MTP*")</f>
-        <v/>
-      </c>
+          <t>• Method: audited the master test plans against the actual product code to find behaviour with no test case (functional gaps), then cross-referenced each against engineering PR-run tests so QA does not duplicate eng work.</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="n"/>
       <c r="C4" s="166" t="n"/>
       <c r="D4" s="166" t="n"/>
       <c r="E4" s="166" t="n"/>
       <c r="F4" s="166" t="n"/>
-      <c r="G4" s="166" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="166" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ...of which eng-covered (add to MTP only, do NOT automate)</t>
-        </is>
-      </c>
-      <c r="B5" s="166">
-        <f>COUNTIF('Gap Analysis'!$L:$L,"Add to MTP only*")</f>
-        <v/>
-      </c>
+          <t>• Two outputs: (1) MTP completeness = ALL functional gaps get added to the plan; (2) QA automation backlog = only the gaps eng does NOT already cover.</t>
+        </is>
+      </c>
+      <c r="B5" s="166" t="n"/>
       <c r="C5" s="166" t="n"/>
       <c r="D5" s="166" t="n"/>
       <c r="E5" s="166" t="n"/>
       <c r="F5" s="166" t="n"/>
-      <c r="G5" s="166" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="166" t="inlineStr">
         <is>
-          <t>Output 2: functional gaps to AUTOMATE (QA backlog)</t>
-        </is>
-      </c>
-      <c r="B6" s="166">
-        <f>COUNTIF('Gap Analysis'!$L:$L,"*Automate*")</f>
-        <v/>
-      </c>
+          <t>• New gaps are mostly eng-covered: the majority of functional gaps found in code are already tested by eng at the logic layer -&gt; add to MTP for completeness, but do NOT re-automate. QA new-automation shortlist is small (real device/SMS/push/cross-system).</t>
+        </is>
+      </c>
+      <c r="B6" s="166" t="n"/>
       <c r="C6" s="166" t="n"/>
       <c r="D6" s="166" t="n"/>
       <c r="E6" s="166" t="n"/>
       <c r="F6" s="166" t="n"/>
-      <c r="G6" s="166" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="166" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ...of which QA-owned (eng cannot cover)</t>
-        </is>
-      </c>
-      <c r="B7" s="166">
-        <f>COUNTIF('Gap Analysis'!$L:$L,"*QA-owned*")</f>
-        <v/>
-      </c>
+          <t>• Existing MTP backlog is the opposite: automatable-not-built existing cases are overwhelmingly UI / end-to-end journeys that eng unit tests do NOT cover -&gt; this backlog genuinely needs QA automation (not duplicative of eng).</t>
+        </is>
+      </c>
+      <c r="B7" s="166" t="n"/>
       <c r="C7" s="166" t="n"/>
       <c r="D7" s="166" t="n"/>
       <c r="E7" s="166" t="n"/>
       <c r="F7" s="166" t="n"/>
-      <c r="G7" s="166" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="166" t="inlineStr">
         <is>
-          <t>Dev: unit-test-coverage gaps</t>
-        </is>
-      </c>
-      <c r="B8" s="166">
-        <f>COUNTIF('Gap Analysis'!$L:$L,"Dev:*")</f>
-        <v/>
-      </c>
+          <t>• Net: eng-overlap savings land almost entirely on the NEW gaps, not the existing backlog. Manual-only (red) items stay manual regardless of framework.</t>
+        </is>
+      </c>
+      <c r="B8" s="166" t="n"/>
       <c r="C8" s="166" t="n"/>
       <c r="D8" s="166" t="n"/>
       <c r="E8" s="166" t="n"/>
       <c r="F8" s="166" t="n"/>
-      <c r="G8" s="166" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="166" t="inlineStr">
         <is>
-          <t>Cross-cutting: reconcile plan/code</t>
-        </is>
-      </c>
-      <c r="B9" s="166">
-        <f>COUNTIF('Gap Analysis'!$L:$L,"Reconcile*")</f>
-        <v/>
-      </c>
+          <t>• All eng-coverage tags are best-guess from reading eng test structure, not verified line coverage - confirm the Partial items with the dev teams.</t>
+        </is>
+      </c>
+      <c r="B9" s="166" t="n"/>
       <c r="C9" s="166" t="n"/>
       <c r="D9" s="166" t="n"/>
       <c r="E9" s="166" t="n"/>
       <c r="F9" s="166" t="n"/>
-      <c r="G9" s="166" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="166" t="inlineStr">
-        <is>
-          <t>Total Gap Analysis rows</t>
-        </is>
-      </c>
-      <c r="B10" s="166">
-        <f>COUNTA('Gap Analysis'!$A$2:$A$1000)</f>
-        <v/>
-      </c>
+      <c r="A10" s="166" t="inlineStr"/>
+      <c r="B10" s="166" t="n"/>
       <c r="C10" s="166" t="n"/>
       <c r="D10" s="166" t="n"/>
       <c r="E10" s="166" t="n"/>
       <c r="F10" s="166" t="n"/>
-      <c r="G10" s="166" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="166" t="n"/>
+      <c r="A11" s="177" t="inlineStr">
+        <is>
+          <t>OUTPUTS (from Gap Analysis)</t>
+        </is>
+      </c>
       <c r="B11" s="166" t="n"/>
       <c r="C11" s="166" t="n"/>
       <c r="D11" s="166" t="n"/>
       <c r="E11" s="166" t="n"/>
       <c r="F11" s="166" t="n"/>
-      <c r="G11" s="166" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="166" t="inlineStr">
         <is>
-          <t>COVERAGE TRACKER — automation of existing MTP cases</t>
-        </is>
-      </c>
-      <c r="B12" s="166" t="inlineStr"/>
+          <t>Output 1: functional gaps to ADD to MTP</t>
+        </is>
+      </c>
+      <c r="B12" s="166">
+        <f>COUNTIF('Gap Analysis'!$L:$L,"Add to MTP*")</f>
+        <v/>
+      </c>
       <c r="C12" s="166" t="n"/>
       <c r="D12" s="166" t="n"/>
       <c r="E12" s="166" t="n"/>
       <c r="F12" s="166" t="n"/>
-      <c r="G12" s="166" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="168" t="inlineStr">
-        <is>
-          <t>Surface</t>
-        </is>
-      </c>
-      <c r="B13" s="168" t="inlineStr">
-        <is>
-          <t>Automated (built)</t>
-        </is>
-      </c>
-      <c r="C13" s="168" t="inlineStr">
-        <is>
-          <t>Automatable (not built)</t>
-        </is>
-      </c>
-      <c r="D13" s="168" t="inlineStr">
-        <is>
-          <t>Manual only</t>
-        </is>
-      </c>
-      <c r="E13" s="168" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="F13" s="168" t="inlineStr">
-        <is>
-          <t>% Automated</t>
-        </is>
-      </c>
-      <c r="G13" s="168" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
+      <c r="A13" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ...of which eng-covered (add to MTP only, do NOT automate)</t>
+        </is>
+      </c>
+      <c r="B13" s="166">
+        <f>COUNTIF('Gap Analysis'!$L:$L,"Add to MTP only*")</f>
+        <v/>
+      </c>
+      <c r="C13" s="166" t="n"/>
+      <c r="D13" s="166" t="n"/>
+      <c r="E13" s="166" t="n"/>
+      <c r="F13" s="166" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="166" t="inlineStr">
         <is>
-          <t>Personal ID Tests</t>
+          <t>Output 2: functional gaps to AUTOMATE (QA backlog)</t>
         </is>
       </c>
       <c r="B14" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A14,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <f>COUNTIF('Gap Analysis'!$L:$L,"*Automate*")</f>
         <v/>
       </c>
-      <c r="C14" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A14,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
-        <v/>
-      </c>
-      <c r="D14" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A14,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
-        <v/>
-      </c>
-      <c r="E14" s="166">
-        <f>B14+C14+D14</f>
-        <v/>
-      </c>
-      <c r="F14" s="174">
-        <f>IF(E14&gt;0,B14/E14,0)</f>
-        <v/>
-      </c>
-      <c r="G14" s="166" t="inlineStr"/>
+      <c r="C14" s="166" t="n"/>
+      <c r="D14" s="166" t="n"/>
+      <c r="E14" s="166" t="n"/>
+      <c r="F14" s="166" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="166" t="inlineStr">
         <is>
-          <t>Integration Tests (Connect)</t>
+          <t xml:space="preserve">   ...of which QA-owned (eng cannot cover)</t>
         </is>
       </c>
       <c r="B15" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A15,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <f>COUNTIF('Gap Analysis'!$L:$L,"*QA-owned*")</f>
         <v/>
       </c>
-      <c r="C15" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A15,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
-        <v/>
-      </c>
-      <c r="D15" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A15,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
-        <v/>
-      </c>
-      <c r="E15" s="166">
-        <f>B15+C15+D15</f>
-        <v/>
-      </c>
-      <c r="F15" s="174">
-        <f>IF(E15&gt;0,B15/E15,0)</f>
-        <v/>
-      </c>
-      <c r="G15" s="166" t="inlineStr"/>
+      <c r="C15" s="166" t="n"/>
+      <c r="D15" s="166" t="n"/>
+      <c r="E15" s="166" t="n"/>
+      <c r="F15" s="166" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="166" t="inlineStr">
         <is>
-          <t>Connect Landing Page</t>
+          <t>Dev: unit-test-coverage gaps</t>
         </is>
       </c>
       <c r="B16" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A16,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <f>COUNTIF('Gap Analysis'!$L:$L,"Dev:*")</f>
         <v/>
       </c>
-      <c r="C16" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A16,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
-        <v/>
-      </c>
-      <c r="D16" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A16,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
-        <v/>
-      </c>
-      <c r="E16" s="166">
-        <f>B16+C16+D16</f>
-        <v/>
-      </c>
-      <c r="F16" s="174">
-        <f>IF(E16&gt;0,B16/E16,0)</f>
-        <v/>
-      </c>
-      <c r="G16" s="166" t="inlineStr"/>
+      <c r="C16" s="166" t="n"/>
+      <c r="D16" s="166" t="n"/>
+      <c r="E16" s="166" t="n"/>
+      <c r="F16" s="166" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="166" t="inlineStr">
         <is>
-          <t>Connect messaging</t>
+          <t>Cross-cutting: reconcile plan/code</t>
         </is>
       </c>
       <c r="B17" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A17,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <f>COUNTIF('Gap Analysis'!$L:$L,"Reconcile*")</f>
         <v/>
       </c>
-      <c r="C17" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A17,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
+      <c r="C17" s="166" t="n"/>
+      <c r="D17" s="166" t="n"/>
+      <c r="E17" s="166" t="n"/>
+      <c r="F17" s="166" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="166" t="inlineStr"/>
+      <c r="B18" s="166" t="n"/>
+      <c r="C18" s="166" t="n"/>
+      <c r="D18" s="166" t="n"/>
+      <c r="E18" s="166" t="n"/>
+      <c r="F18" s="166" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="177" t="inlineStr">
+        <is>
+          <t>COVERAGE TRACKER — automation of existing MTP cases</t>
+        </is>
+      </c>
+      <c r="B19" s="166" t="n"/>
+      <c r="C19" s="166" t="n"/>
+      <c r="D19" s="166" t="n"/>
+      <c r="E19" s="166" t="n"/>
+      <c r="F19" s="166" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="168" t="inlineStr">
+        <is>
+          <t>Surface</t>
+        </is>
+      </c>
+      <c r="B20" s="168" t="inlineStr">
+        <is>
+          <t>Automated (built)</t>
+        </is>
+      </c>
+      <c r="C20" s="168" t="inlineStr">
+        <is>
+          <t>Automatable (not built)</t>
+        </is>
+      </c>
+      <c r="D20" s="168" t="inlineStr">
+        <is>
+          <t>Manual only</t>
+        </is>
+      </c>
+      <c r="E20" s="168" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="F20" s="168" t="inlineStr">
+        <is>
+          <t>% Automated</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="166" t="inlineStr">
+        <is>
+          <t>Personal ID Tests</t>
+        </is>
+      </c>
+      <c r="B21" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A21,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
         <v/>
       </c>
-      <c r="D17" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A17,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
+      <c r="C21" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A21,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
         <v/>
       </c>
-      <c r="E17" s="166">
-        <f>B17+C17+D17</f>
+      <c r="D21" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A21,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
         <v/>
       </c>
-      <c r="F17" s="174">
-        <f>IF(E17&gt;0,B17/E17,0)</f>
+      <c r="E21" s="166">
+        <f>B21+C21+D21</f>
         <v/>
       </c>
-      <c r="G17" s="166" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="166" t="inlineStr">
-        <is>
-          <t>Connect Notifications</t>
-        </is>
-      </c>
-      <c r="B18" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A18,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
-        <v/>
-      </c>
-      <c r="C18" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A18,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
-        <v/>
-      </c>
-      <c r="D18" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A18,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
-        <v/>
-      </c>
-      <c r="E18" s="166">
-        <f>B18+C18+D18</f>
-        <v/>
-      </c>
-      <c r="F18" s="174">
-        <f>IF(E18&gt;0,B18/E18,0)</f>
-        <v/>
-      </c>
-      <c r="G18" s="166" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="166" t="inlineStr">
-        <is>
-          <t>Connect worker History</t>
-        </is>
-      </c>
-      <c r="B19" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A19,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
-        <v/>
-      </c>
-      <c r="C19" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A19,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
-        <v/>
-      </c>
-      <c r="D19" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A19,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
-        <v/>
-      </c>
-      <c r="E19" s="166">
-        <f>B19+C19+D19</f>
-        <v/>
-      </c>
-      <c r="F19" s="174">
-        <f>IF(E19&gt;0,B19/E19,0)</f>
-        <v/>
-      </c>
-      <c r="G19" s="166" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="166" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Case List map </t>
-        </is>
-      </c>
-      <c r="B20" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A20,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
-        <v/>
-      </c>
-      <c r="C20" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A20,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
-        <v/>
-      </c>
-      <c r="D20" s="166">
-        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A20,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
-        <v/>
-      </c>
-      <c r="E20" s="166">
-        <f>B20+C20+D20</f>
-        <v/>
-      </c>
-      <c r="F20" s="174">
-        <f>IF(E20&gt;0,B20/E20,0)</f>
-        <v/>
-      </c>
-      <c r="G20" s="166" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="175" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B21" s="175">
-        <f>SUM(B14:B20)</f>
-        <v/>
-      </c>
-      <c r="C21" s="175">
-        <f>SUM(C14:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="175">
-        <f>SUM(D14:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="175">
-        <f>SUM(E14:E20)</f>
-        <v/>
-      </c>
-      <c r="F21" s="176">
+      <c r="F21" s="174">
         <f>IF(E21&gt;0,B21/E21,0)</f>
         <v/>
       </c>
-      <c r="G21" s="175" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="166" t="inlineStr">
+        <is>
+          <t>Integration Tests (Connect)</t>
+        </is>
+      </c>
+      <c r="B22" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A22,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <v/>
+      </c>
+      <c r="C22" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A22,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D22" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A22,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E22" s="166">
+        <f>B22+C22+D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="174">
+        <f>IF(E22&gt;0,B22/E22,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="180" t="inlineStr">
-        <is>
-          <t>EXISTING automatable-not-built cases — do they need automating?</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
+      <c r="A23" s="166" t="inlineStr">
+        <is>
+          <t>Connect Landing Page</t>
+        </is>
+      </c>
+      <c r="B23" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A23,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <v/>
+      </c>
+      <c r="C23" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A23,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D23" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A23,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E23" s="166">
+        <f>B23+C23+D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="174">
+        <f>IF(E23&gt;0,B23/E23,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="166" t="inlineStr">
         <is>
+          <t>Connect messaging</t>
+        </is>
+      </c>
+      <c r="B24" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A24,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <v/>
+      </c>
+      <c r="C24" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A24,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D24" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A24,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E24" s="166">
+        <f>B24+C24+D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="174">
+        <f>IF(E24&gt;0,B24/E24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="166" t="inlineStr">
+        <is>
+          <t>Connect Notifications</t>
+        </is>
+      </c>
+      <c r="B25" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A25,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <v/>
+      </c>
+      <c r="C25" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A25,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D25" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A25,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E25" s="166">
+        <f>B25+C25+D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="174">
+        <f>IF(E25&gt;0,B25/E25,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="166" t="inlineStr">
+        <is>
+          <t>Connect worker History</t>
+        </is>
+      </c>
+      <c r="B26" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A26,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <v/>
+      </c>
+      <c r="C26" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A26,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D26" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A26,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E26" s="166">
+        <f>B26+C26+D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="174">
+        <f>IF(E26&gt;0,B26/E26,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Case List map </t>
+        </is>
+      </c>
+      <c r="B27" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A27,'Automation (existing MTP)'!$D:$D,"🟢*")</f>
+        <v/>
+      </c>
+      <c r="C27" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A27,'Automation (existing MTP)'!$D:$D,"🟡*")</f>
+        <v/>
+      </c>
+      <c r="D27" s="166">
+        <f>COUNTIFS('Automation (existing MTP)'!$B:$B,$A27,'Automation (existing MTP)'!$D:$D,"🔴*")</f>
+        <v/>
+      </c>
+      <c r="E27" s="166">
+        <f>B27+C27+D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="174">
+        <f>IF(E27&gt;0,B27/E27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="175" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="175">
+        <f>SUM(B21:B27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="175">
+        <f>SUM(C21:C27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="175">
+        <f>SUM(D21:D27)</f>
+        <v/>
+      </c>
+      <c r="E28" s="175">
+        <f>SUM(E21:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="176">
+        <f>IF(E28&gt;0,B28/E28,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="166" t="inlineStr"/>
+      <c r="B29" s="166" t="n"/>
+      <c r="C29" s="166" t="n"/>
+      <c r="D29" s="166" t="n"/>
+      <c r="E29" s="166" t="n"/>
+      <c r="F29" s="166" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="177" t="inlineStr">
+        <is>
+          <t>EXISTING automatable-not-built cases — do they need automating?</t>
+        </is>
+      </c>
+      <c r="B30" s="166" t="n"/>
+      <c r="C30" s="166" t="n"/>
+      <c r="D30" s="166" t="n"/>
+      <c r="E30" s="166" t="n"/>
+      <c r="F30" s="166" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="166" t="inlineStr">
+        <is>
           <t>QA-owned (UI/e2e - need automating)</t>
         </is>
       </c>
-      <c r="B24">
+      <c r="B31" s="166">
         <f>COUNTIF('Automation (existing MTP)'!$G:$G,"QA-owned (UI*")</f>
         <v/>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="166" t="inlineStr">
+      <c r="C31" s="166" t="n"/>
+      <c r="D31" s="166" t="n"/>
+      <c r="E31" s="166" t="n"/>
+      <c r="F31" s="166" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="166" t="inlineStr">
         <is>
           <t>Likely already eng-covered (confirm - may NOT need automating)</t>
         </is>
       </c>
-      <c r="B25">
+      <c r="B32" s="166">
         <f>COUNTIF('Automation (existing MTP)'!$G:$G,"Partial*")</f>
         <v/>
       </c>
+      <c r="C32" s="166" t="n"/>
+      <c r="D32" s="166" t="n"/>
+      <c r="E32" s="166" t="n"/>
+      <c r="F32" s="166" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>